<commit_message>
Rework brand pages to standardised conditional H2 template
Brand collections now use H1 '[Brand] Golf Weights' with a uniform,
stock-conditional H2 set ([Brand] Putter/Driver/Fairway/Iron Weights,
Weight Kits, Shaft Adapters, Tools) ordered by search demand per brand.
Bespoke content (charts, how-tos, model lists) moves to a new 'Text
block further down the page' column; adapter collections likewise carry
their settings charts in the text-block column. Read Me updated with
the template rules and the real-H2-headings-in-text-blocks requirement.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016qLKXS24xJWKHvQuj4G8VR
</commit_message>
<xml_diff>
--- a/deliverables/golfweights/GolfWeights_SEO_Implementation_Sheet.xlsx
+++ b/deliverables/golfweights/GolfWeights_SEO_Implementation_Sheet.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -644,45 +644,69 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>The H2 suggestions match the new page template: each H2 introduces a section/product carousel on the page (e.g. 'TaylorMade Driver Weights' above the driver products). Add them in the order given. On product pages they are ordinary content headings (fitment list, weight options, how-to).</t>
+          <t>The H2 suggestions match the new page template: each H2 introduces a section/product carousel on the page (e.g. 'TaylorMade Driver Weights' above the driver products). Add them in the order given — the first section is that brand's biggest seller in search. Only build a section if you actually stock those products (the lists here already reflect current stock); never leave an empty section on the page. On product pages the H2s are ordinary content headings (fitment list, weight options, how-to).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Internal links</t>
+          <t>Brand page template</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>On the 'Internal Links' tab, each row lists the links to add ON that page. 'Links to' is the destination; 'Anchor text' is the exact clickable wording. Add them naturally in the page's intro or description text.</t>
+          <t>Every brand collection follows the same pattern: H1 '[Brand] Golf Weights', then conditional H2 sections ([Brand] Putter/Driver/Fairway/Iron Weights, [Brand] Weight Kits, [Brand] Shaft Adapters) with a product carousel under each. Brand-specific extras (charts, how-to guides, model lists) go in a text block further down — see the next row.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="2" t="n"/>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Text blocks</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>The 'Text block further down' column lists extra content for the bottom of the page. IMPORTANT: headings inside text blocks must be set as real Heading 2 / Heading 3 in the Shopify editor (the paragraph-style dropdown), NOT just bold text — Google only counts proper headings. Charts must be real text tables, not images.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>Internal links</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>On the 'Internal Links' tab, each row lists the links to add ON that page. 'Links to' is the destination; 'Anchor text' is the exact clickable wording. Add them naturally in the page's intro or description text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>Delivery claims used</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Descriptions use: UK stock · same-day dispatch before 1pm · free delivery over £40. If any of these change, let us know and we'll update the wording.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Questions?</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Anything unclear — ask before publishing. It's much easier to fix in this sheet than after Google has re-crawled the site.</t>
         </is>
@@ -699,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M270"/>
+  <dimension ref="A1:N270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -708,13 +732,14 @@
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="58" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -779,6 +804,11 @@
         </is>
       </c>
       <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Text block further down the page (use real H2/H3 headings)</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>Remove / avoid on this page</t>
         </is>
@@ -802,6 +832,7 @@
       <c r="K2" s="6" t="n"/>
       <c r="L2" s="6" t="n"/>
       <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -860,7 +891,8 @@
         </is>
       </c>
       <c r="L3" s="8" t="n"/>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="M3" s="8" t="n"/>
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Nothing to remove — but note: this is the ONLY page allowed to target 'golf weights' / 'golf club weights'. Six of your pages currently compete for that phrase; the other five are de-optimised in this sheet.</t>
         </is>
@@ -884,6 +916,7 @@
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="6" t="n"/>
       <c r="M4" s="6" t="n"/>
+      <c r="N4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -934,7 +967,8 @@
       <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="n"/>
+      <c r="N5" s="8" t="inlineStr">
         <is>
           <t>Stop targeting 'drivers' on its own — this page can't outrank club retailers for it and it's the wrong buyer. Every heading pairs 'driver' with 'weights'.</t>
         </is>
@@ -989,7 +1023,8 @@
       <c r="J6" s="8" t="n"/>
       <c r="K6" s="8" t="n"/>
       <c r="L6" s="8" t="n"/>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="M6" s="8" t="n"/>
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Stop targeting 'putter' / 'golf putter' on their own (currently position 55 — wrong intent, unwinnable). This page — not any product page — owns 'putter weights'; the Scotty product page competing for it is being retitled in this sheet.</t>
         </is>
@@ -1040,7 +1075,8 @@
       <c r="J7" s="8" t="n"/>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="inlineStr">
+      <c r="M7" s="8" t="n"/>
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>Stop targeting 'fairway woods' on its own (currently position 50 — people searching that want to buy a club, not a weight).</t>
         </is>
@@ -1091,7 +1127,8 @@
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
       <c r="L8" s="8" t="n"/>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="M8" s="8" t="n"/>
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>Don't target 'hybrids' or 'hybrid golf clubs' on their own — headings always pair 'hybrid' with 'weights'.</t>
         </is>
@@ -1146,7 +1183,8 @@
       <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
-      <c r="M9" s="8" t="inlineStr">
+      <c r="M9" s="8" t="n"/>
+      <c r="N9" s="8" t="inlineStr">
         <is>
           <t>This page currently ranks for 'golf weights' (one of the six competing pages) — remove that phrase from its title and copy; keep it strictly about IRON weights.</t>
         </is>
@@ -1197,7 +1235,8 @@
       <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
       <c r="L10" s="8" t="n"/>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="M10" s="8" t="n"/>
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>Must NOT target 'golf weights' — the homepage owns that phrase and this page is one of the six currently competing for it. Keep the framing as a 'shop all' catalogue page.</t>
         </is>
@@ -1221,6 +1260,7 @@
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="6" t="n"/>
       <c r="M11" s="6" t="n"/>
+      <c r="N11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1240,7 +1280,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Scotty Cameron Putter Weights, Kits &amp; Tools | Golf Weights</t>
+          <t>Scotty Cameron Golf Weights | Putter Weights, Kits &amp; Tools</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1250,14 +1290,14 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
+          <t>Scotty Cameron Golf Weights</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
           <t>Scotty Cameron Putter Weights</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Scotty Cameron Weights by Model (Newport, Phantom &amp; Fastback)</t>
-        </is>
-      </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
           <t>Scotty Cameron Weight Kits</t>
@@ -1268,20 +1308,17 @@
           <t>Scotty Cameron Weight Tools &amp; Wrenches</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Scotty Cameron Putter Weight Chart</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>How to Change Scotty Cameron Weights</t>
-        </is>
-      </c>
+      <c r="J12" s="8" t="n"/>
+      <c r="K12" s="8" t="n"/>
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="inlineStr">
         <is>
-          <t>Stop targeting 'Scotty Cameron' on its own (currently position 39 — you can't outrank Scotty and the big retailers, and those searchers want a putter, not weights). Every heading pairs the brand with 'weights'. This page already ranks #2 for 'scotty cameron putter weights' — it is the template for all the other brand pages.</t>
+          <t>Add as proper H2 headings in a text block: 'Scotty Cameron Putter Weight Chart' (weights by model, 10g–40g, as a real table) and 'How to Change Scotty Cameron Weights' (short steps, link the weight tool). In the intro copy, name the model families — Newport, Phantom, Fastback, Squareback.</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>Stop targeting 'Scotty Cameron' on its own (currently position 39 — you can't outrank Scotty and the big retailers, and those searchers want a putter, not weights). This page already ranks #2 for 'scotty cameron putter weights' — keep that phrase in the title and first H2 exactly as written.</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1340,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>TaylorMade Golf Weights &amp; Kits | Driver &amp; Spider Putter Weights</t>
+          <t>TaylorMade Golf Weights | Driver &amp; Spider Putter Weights</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1323,12 +1360,12 @@
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>TaylorMade Spider &amp; TP Putter Weights</t>
+          <t>TaylorMade Putter Weights</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>TaylorMade Fairway &amp; Hybrid Weights</t>
+          <t>TaylorMade Fairway Wood Weights</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
@@ -1341,10 +1378,19 @@
           <t>TaylorMade Shaft Adapters</t>
         </is>
       </c>
-      <c r="L13" s="8" t="n"/>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>TaylorMade Wrenches &amp; Tools</t>
+        </is>
+      </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
-          <t>Remove bare model names as targets (e.g. 'TaylorMade Qi10' alone) — model phrases belong on product pages, always with 'weights' added. This page currently competes for 'golf weights' — keep it strictly TaylorMade.</t>
+          <t>Optional H3 under the putter section: 'TaylorMade Spider Putter Weights' — the Spider phrase carries most of the putter demand (~740/mo US). In the intro copy, name the ranges — Qi10, Qi35, Stealth, SIM, M-Series, BRNR, Spider, TP.</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>Remove bare model names as targets (e.g. 'TaylorMade Qi10' alone) — model phrases belong on product pages, always with 'weights' added. Keep 'golf weights' brand-qualified (always 'TaylorMade golf weights', never standalone) — this page is one of the six currently competing with the homepage.</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1412,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Odyssey Putter Weights &amp; Weight Kits | Ai-ONE, Jailbird &amp; White Hot</t>
+          <t>Odyssey Golf Weights | Putter Weights &amp; Weight Kits</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1376,34 +1422,35 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
+          <t>Odyssey Golf Weights</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
           <t>Odyssey Putter Weights</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Odyssey Ai-ONE Weights</t>
-        </is>
-      </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Odyssey Stroke Lab &amp; White Hot Weights</t>
+          <t>Odyssey Weight Kits</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Odyssey Jailbird &amp; Toulon Weights</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Odyssey Weight Kits</t>
-        </is>
-      </c>
+          <t>Odyssey Weight Tools &amp; Wrenches</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="inlineStr">
         <is>
-          <t>This page ALONE owns 'Odyssey putter weights' — two product pages currently compete with it for that phrase and are being retitled to model-only names in this sheet.</t>
+          <t>In the intro copy, name the model families — Ai-ONE, Jailbird, White Hot, Stroke Lab, Toulon.</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>This page ALONE owns 'Odyssey putter weights' — keep that phrase in the title and first H2. Two product pages currently compete with it for that phrase and are being retitled to model-only names in this sheet.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1472,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>PXG Golf Weights &amp; Weight Kits | Driver, Iron &amp; Putter</t>
+          <t>PXG Golf Weights | Driver, Iron &amp; Putter Weight Kits</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -1440,7 +1487,7 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>PXG Driver Weights (Black Ops &amp; Gen Series)</t>
+          <t>PXG Driver Weights</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -1450,7 +1497,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>PXG Putter Weights (Battle Ready)</t>
+          <t>PXG Putter Weights</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -1460,12 +1507,17 @@
       </c>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>PXG Weight Chart</t>
+          <t>PXG Shaft Adapters</t>
         </is>
       </c>
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="8" t="inlineStr">
         <is>
+          <t>Optional H2 in a text block: 'PXG Weight Chart' — there are chart searches for PXG (~80/mo US). In the intro copy, name Black Ops, the Gen series and Battle Ready.</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
           <t>Stop targeting 'PXG' on its own (currently position 19 — unwinnable, wrong intent). Every heading pairs PXG with 'weights'.</t>
         </is>
       </c>
@@ -1488,7 +1540,7 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Callaway Golf Weights &amp; Kits | Driver &amp; Fairway Wood Weights</t>
+          <t>Callaway Golf Weights | Driver &amp; Fairway Wood Weights</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1513,7 +1565,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Callaway Apex Iron &amp; Hybrid Weights</t>
+          <t>Callaway Hybrid Weights</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -1529,6 +1581,11 @@
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="8" t="inlineStr">
         <is>
+          <t>In the intro copy, name the ranges — Elyte, Paradym, Rogue, Mavrik, Epic, Apex.</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
           <t>Don't target bare model names ('Callaway Paradym' alone) — model phrases live on product pages with 'weights' added.</t>
         </is>
       </c>
@@ -1551,7 +1608,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Ping Golf Weights &amp; Kits | Driver &amp; Iron Weights (G425–G440)</t>
+          <t>Ping Golf Weights | Driver &amp; Iron Weights (G425–G440)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1566,22 +1623,22 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Ping Driver Weights (G30–G440)</t>
+          <t>Ping Driver Weights</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>Ping Fairway &amp; Hybrid Weights</t>
+          <t>Ping Fairway Wood Weights</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Ping Iron Weight Replacements</t>
+          <t>Ping Iron Weights</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>Ping Putter Weights (Vault)</t>
+          <t>Ping Putter Weights</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr">
@@ -1589,10 +1646,19 @@
           <t>Ping Weight Kits</t>
         </is>
       </c>
-      <c r="L17" s="8" t="n"/>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Ping Shaft Adapters</t>
+        </is>
+      </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
-          <t>Keep the iron weight replacement content — this page already ranks #1 for 'ping iron weight replacement'. Don't target bare model names ('Ping G425 driver' alone).</t>
+          <t>Move the existing 'ping iron weight replacement' copy under the Ping Iron Weights section — do not delete or rewrite it (it ranks #1). Optional H2: 'Ping G-Series Weights by Generation (G30–G440)'. Cross-sell the Ping Vault putter wrench in the putter section.</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>Don't target bare model names ('Ping G425 driver' alone). KEEP the iron weight replacement copy — this page ranks #1 for 'ping iron weight replacement'.</t>
         </is>
       </c>
     </row>
@@ -1614,12 +1680,12 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Titleist Golf Weights &amp; Kits | SureFit Driver &amp; Fairway Weights</t>
+          <t>Titleist Golf Weights | SureFit Driver Weights &amp; Kits</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Aftermarket Titleist SureFit weights and weight kits for GT, TSR, TS and 913–917 drivers and fairways. UK stock — same-day dispatch before 1pm and free delivery over £40.</t>
+          <t>Titleist SureFit weights and weight kits for GT, TSR, TS and 913–917 drivers and fairways. UK stock — same-day dispatch before 1pm and free delivery over £40.</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1629,29 +1695,38 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Titleist Driver Weights (GT, TSR &amp; TS)</t>
+          <t>Titleist Driver Weights</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Titleist Fairway &amp; Hybrid Weights</t>
+          <t>Titleist Fairway Wood Weights</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>Titleist SureFit Weight Kits</t>
+          <t>Titleist Hybrid Weights</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>Titleist Shaft Adapters &amp; SureFit Chart</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="n"/>
+          <t>Titleist Weight Kits</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Titleist Shaft Adapters</t>
+        </is>
+      </c>
       <c r="L18" s="8" t="n"/>
       <c r="M18" s="8" t="inlineStr">
         <is>
-          <t>This page currently competes for 'golf weights' — keep it strictly Titleist. Weight-settings searches are big for Titleist: cross-link the adapter page's SureFit chart prominently.</t>
+          <t>Optional H2 in a text block: 'Titleist Weight Settings (GT &amp; TS)' — settings searches are big for Titleist (e.g. GT3 weight adjustment, ~200/mo US). Cross-link the SureFit chart on the Titleist adapter page prominently.</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>Keep 'golf weights' brand-qualified (always 'Titleist golf weights', never standalone) — this page is one of the six currently competing with the homepage.</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1748,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Cobra Golf Weights | Driver, Fairway &amp; Putter Weights</t>
+          <t>Cobra Golf Weights | Driver &amp; Putter Weights</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1688,17 +1763,17 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Cobra Driver Weights (Darkspeed, Aerojet, LTDx &amp; Radspeed)</t>
+          <t>Cobra Driver Weights</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>Cobra Fairway &amp; Hybrid Weights</t>
+          <t>Cobra Fairway Wood Weights</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Cobra King Putter Weights</t>
+          <t>Cobra Putter Weights</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -1714,6 +1789,11 @@
       <c r="L19" s="8" t="n"/>
       <c r="M19" s="8" t="inlineStr">
         <is>
+          <t>In the intro copy, name the ranges — Darkspeed, DS-Adapt, Aerojet, LTDx, Radspeed, King.</t>
+        </is>
+      </c>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
           <t>Don't target bare model names ('Cobra Aerojet' alone — its product page currently ranks #12 for that, wrong intent; it's being retitled to '...Weights').</t>
         </is>
       </c>
@@ -1751,7 +1831,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Srixon Driver Weights (ZXi &amp; ZX)</t>
+          <t>Srixon Driver Weights</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -1769,7 +1849,12 @@
       <c r="L20" s="8" t="n"/>
       <c r="M20" s="8" t="inlineStr">
         <is>
-          <t>Keep this page light — Srixon's real search demand is shaft adapters, so the adapter link should be prominent (banner-level).</t>
+          <t>Make the Srixon Shaft Adapters link prominent (banner-level) — adapters are Srixon's biggest search cluster.</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>Keep this page light — Srixon's real search demand is shaft adapters.</t>
         </is>
       </c>
     </row>
@@ -1791,44 +1876,41 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Mizuno Putter Weights | M-Craft Weights &amp; Kits</t>
+          <t>Mizuno Golf Weights | ST Driver Weights &amp; Adapters</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Aftermarket Mizuno putter weights for the M-Craft range, plus ST-series driver weights. UK stock — same-day dispatch before 1pm and free delivery over £40.</t>
+          <t>Aftermarket Mizuno weights and shaft adapters for the ST range of drivers. UK stock — same-day dispatch before 1pm and free delivery over £40.</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Mizuno Putter Weights</t>
+          <t>Mizuno Golf Weights</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Mizuno M-Craft Putter Weights</t>
+          <t>Mizuno Driver Weights</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>Mizuno ST Driver Weights</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Mizuno Weight Kits</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
           <t>Mizuno Shaft Adapters</t>
         </is>
       </c>
+      <c r="I21" s="8" t="n"/>
+      <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="inlineStr">
         <is>
-          <t>This page currently competes for 'golf weights' — keep it strictly Mizuno.</t>
+          <t>There IS search demand for 'Mizuno putter weights' (M-Craft, ~10–30/mo UK) but no putter products were found in the catalogue — if you stock M-Craft putter weights, add a 'Mizuno Putter Weights' H2 section and tell us so we can update the targeting.</t>
+        </is>
+      </c>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>Keep 'golf weights' brand-qualified (always 'Mizuno golf weights', never standalone) — this page is one of the six currently competing with the homepage.</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1932,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>LAB Golf Putter Weights | DF &amp; Mezz</t>
+          <t>LAB Golf Weights | Putter Weights for DF &amp; Mezz</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1860,25 +1942,26 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
+          <t>LAB Golf Weights</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
           <t>LAB Golf Putter Weights</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>LAB Golf Weights by Model</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>How LAB Putter Weighting Works</t>
-        </is>
-      </c>
+      <c r="H22" s="8" t="n"/>
       <c r="I22" s="8" t="n"/>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="n"/>
       <c r="M22" s="8" t="inlineStr">
         <is>
+          <t>One intro sentence naming DF and Mezz is enough.</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
           <t>Light page — rising brand. Keep headings paired with 'weights'.</t>
         </is>
       </c>
@@ -1916,7 +1999,7 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Honma T//World Weights</t>
+          <t>Honma Driver Weights</t>
         </is>
       </c>
       <c r="H23" s="8" t="n"/>
@@ -1926,6 +2009,11 @@
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="8" t="inlineStr">
         <is>
+          <t>One intro sentence is enough.</t>
+        </is>
+      </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
           <t>Minimal effort page — negligible search demand. Just apply the title/H1 and move on.</t>
         </is>
       </c>
@@ -1948,7 +2036,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Toulon Design Putter Weights | Golf Weights</t>
+          <t>Toulon Design Golf Weights | Putter Weights &amp; Kits</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -1958,20 +2046,29 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Toulon Design Putter Weights</t>
+          <t>Toulon Design Golf Weights</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Toulon Weights by Collection</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="n"/>
+          <t>Toulon Putter Weights</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Toulon Weight Kits</t>
+        </is>
+      </c>
       <c r="I24" s="8" t="n"/>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="8" t="n"/>
       <c r="M24" s="8" t="inlineStr">
+        <is>
+          <t>One intro sentence naming the 2022 and 2025 collections is enough.</t>
+        </is>
+      </c>
+      <c r="N24" s="8" t="inlineStr">
         <is>
           <t>Minimal effort page — negligible search demand. Just apply the title/H1 and move on.</t>
         </is>
@@ -1995,6 +2092,7 @@
       <c r="K25" s="6" t="n"/>
       <c r="L25" s="6" t="n"/>
       <c r="M25" s="6" t="n"/>
+      <c r="N25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2034,23 +2132,24 @@
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>Adapter Settings &amp; Compatibility Charts</t>
+          <t>Left-Handed Shaft Adapters</t>
         </is>
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>Left-Handed Shaft Adapters</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="inlineStr">
-        <is>
           <t>Torque Wrenches for Fitting</t>
         </is>
       </c>
+      <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="8" t="n"/>
       <c r="M26" s="8" t="inlineStr">
         <is>
+          <t>Add an 'Adapter Settings &amp; Compatibility Charts' H2 section that links to each brand's chart with descriptive anchors ('Titleist SureFit chart', 'Callaway OptiFit chart' etc.).</t>
+        </is>
+      </c>
+      <c r="N26" s="8" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
@@ -2088,33 +2187,26 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>Titleist SureFit Adapter Chart (A•1–D•4 Settings)</t>
+          <t>Titleist Driver Adapters</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>Titleist Driver Adapters</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="inlineStr">
-        <is>
           <t>Titleist Fairway &amp; Hybrid Adapters</t>
         </is>
       </c>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>Which Adapter Fits Your Titleist?</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="inlineStr">
-        <is>
-          <t>You'll Need a Torque Wrench</t>
-        </is>
-      </c>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="8" t="n"/>
+      <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="8" t="inlineStr">
         <is>
-          <t>BIGGEST single opportunity in this whole plan: put the full SureFit settings/compatibility chart ON this page (as a table, not an image). Searches for the chart alone are ~1,400/month in the US and 100/month in the UK with zero competition difficulty.</t>
+          <t>H2 in a text block: 'Titleist SureFit Adapter Chart' — the full A•1–D•4 settings table as REAL TEXT (not an image), plus a which-adapter-fits-which-model list and an FAQ. Searches for this chart alone: ~1,400/mo US, ~100/mo UK, zero competition difficulty.</t>
+        </is>
+      </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>BIGGEST single opportunity in this whole plan — do the chart (see text block column) before anything else on this page.</t>
         </is>
       </c>
     </row>
@@ -2151,29 +2243,26 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>TaylorMade Loft Sleeve Compatibility Chart (M, SIM, Stealth &amp; Qi)</t>
+          <t>TaylorMade Driver Adapters</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>TaylorMade Driver Adapters</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
           <t>TaylorMade Fairway &amp; Hybrid Adapters</t>
         </is>
       </c>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>TaylorMade Adapter Settings Explained</t>
-        </is>
-      </c>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
       <c r="L28" s="8" t="n"/>
       <c r="M28" s="8" t="inlineStr">
         <is>
-          <t>Your adapter product already ranks #3 for 'compatibility chart' searches — move the chart UP to this collection page and have products link to it. Do NOT change this page's unusual web address.</t>
+          <t>H2s in a text block: 'TaylorMade Loft Sleeve Compatibility Chart' (which sleeve fits M-Series / SIM / Stealth / Qi generations, as a real table) and 'TaylorMade Adapter Settings Explained'. Your adapter product already ranks #3 for the compatibility chart — lift the chart UP to this page and have the products link to it.</t>
+        </is>
+      </c>
+      <c r="N28" s="8" t="inlineStr">
+        <is>
+          <t>Do NOT change this page's unusual web address.</t>
         </is>
       </c>
     </row>
@@ -2210,29 +2299,26 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>Callaway OptiFit Settings Chart</t>
+          <t>Callaway Driver Adapters</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>Callaway Driver Adapters</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
           <t>Callaway Fairway &amp; Hybrid Adapters</t>
         </is>
       </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>Which Adapter Fits Your Callaway?</t>
-        </is>
-      </c>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
       <c r="M29" s="8" t="inlineStr">
         <is>
-          <t>Add the OptiFit settings chart on-page — 'callaway adapter settings' is ~500/month in the US.</t>
+          <t>H2 in a text block: 'Callaway OptiFit Settings Chart' as a real table — 'callaway adapter settings' is ~500/mo in the US.</t>
+        </is>
+      </c>
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2269,29 +2355,26 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Ping Adapter Compatibility by Generation (G400–G440)</t>
+          <t>Ping Driver Adapters</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>Ping Driver Adapters</t>
-        </is>
-      </c>
-      <c r="I30" s="8" t="inlineStr">
-        <is>
           <t>Ping Fairway &amp; Hybrid Adapters</t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
-        <is>
-          <t>Ping Adapter Settings Chart</t>
-        </is>
-      </c>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="8" t="n"/>
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="8" t="n"/>
       <c r="M30" s="8" t="inlineStr">
         <is>
-          <t>Add the generation compatibility table (which adapter fits G400/G410/G425/G430/G440).</t>
+          <t>H2 in a text block: 'Ping Adapter Compatibility by Generation' — a table of which adapter (Gen 1/2/3) fits G400 / G410 / G425 / G430 / G440.</t>
+        </is>
+      </c>
+      <c r="N30" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2328,24 +2411,25 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Cobra Adapter Loft Chart</t>
+          <t>Cobra Driver Adapters</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>Cobra Driver Adapters</t>
-        </is>
-      </c>
-      <c r="I31" s="8" t="inlineStr">
-        <is>
           <t>Cobra Fairway Adapters</t>
         </is>
       </c>
+      <c r="I31" s="8" t="n"/>
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="8" t="n"/>
       <c r="M31" s="8" t="inlineStr">
         <is>
+          <t>Light chart section: 'Cobra Adapter Loft Chart' H2 with a settings table.</t>
+        </is>
+      </c>
+      <c r="N31" s="8" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
@@ -2383,24 +2467,25 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>PXG Adapter Settings Chart</t>
+          <t>PXG Driver Adapters</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>PXG Driver Adapters</t>
-        </is>
-      </c>
-      <c r="I32" s="8" t="inlineStr">
-        <is>
           <t>PXG Hybrid Adapters</t>
         </is>
       </c>
+      <c r="I32" s="8" t="n"/>
       <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
       <c r="L32" s="8" t="n"/>
       <c r="M32" s="8" t="inlineStr">
         <is>
+          <t>Light chart section: 'PXG Adapter Settings Chart' H2 with a settings table.</t>
+        </is>
+      </c>
+      <c r="N32" s="8" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
@@ -2438,20 +2523,21 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Srixon Adapter Settings</t>
-        </is>
-      </c>
-      <c r="H33" s="8" t="inlineStr">
-        <is>
           <t>Srixon Driver Adapters</t>
         </is>
       </c>
+      <c r="H33" s="8" t="n"/>
       <c r="I33" s="8" t="n"/>
       <c r="J33" s="8" t="n"/>
       <c r="K33" s="8" t="n"/>
       <c r="L33" s="8" t="n"/>
       <c r="M33" s="8" t="inlineStr">
         <is>
+          <t>Modest chart section: 'Srixon Adapter Settings' H2 with a settings table.</t>
+        </is>
+      </c>
+      <c r="N33" s="8" t="inlineStr">
+        <is>
           <t>Srixon's best search cluster is adapters (not weights) — this page leads the Srixon effort.</t>
         </is>
       </c>
@@ -2497,7 +2583,8 @@
       <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
       <c r="L34" s="8" t="n"/>
-      <c r="M34" s="8" t="inlineStr">
+      <c r="M34" s="8" t="n"/>
+      <c r="N34" s="8" t="inlineStr">
         <is>
           <t>Minimal effort — apply the title/H1 and move on.</t>
         </is>
@@ -2544,7 +2631,8 @@
       <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
       <c r="L35" s="8" t="n"/>
-      <c r="M35" s="8" t="inlineStr">
+      <c r="M35" s="8" t="n"/>
+      <c r="N35" s="8" t="inlineStr">
         <is>
           <t>Minimal effort — apply the title/H1 and move on.</t>
         </is>
@@ -2586,16 +2674,17 @@
           <t>LH Adapters by Brand</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr">
-        <is>
-          <t>Adapter Settings &amp; Charts</t>
-        </is>
-      </c>
+      <c r="H36" s="8" t="n"/>
       <c r="I36" s="8" t="n"/>
       <c r="J36" s="8" t="n"/>
       <c r="K36" s="8" t="n"/>
       <c r="L36" s="8" t="n"/>
       <c r="M36" s="8" t="inlineStr">
+        <is>
+          <t>Short intro plus a per-brand list of what's available left-handed.</t>
+        </is>
+      </c>
+      <c r="N36" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2619,6 +2708,7 @@
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="6" t="n"/>
       <c r="M37" s="6" t="n"/>
+      <c r="N37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2681,7 +2771,8 @@
           <t>More Brands</t>
         </is>
       </c>
-      <c r="M38" s="8" t="inlineStr">
+      <c r="M38" s="8" t="n"/>
+      <c r="N38" s="8" t="inlineStr">
         <is>
           <t>Do NOT change this page's web address (the '-1' on the end must stay). Per-brand kit searches are strong — the brand H2 sections above each need their own product carousel.</t>
         </is>
@@ -2740,7 +2831,8 @@
       </c>
       <c r="K39" s="8" t="n"/>
       <c r="L39" s="8" t="n"/>
-      <c r="M39" s="8" t="inlineStr">
+      <c r="M39" s="8" t="n"/>
+      <c r="N39" s="8" t="inlineStr">
         <is>
           <t>Your T25 universal wrench already ranks #3–4 for 'golf torque wrench' searches — this collection consolidates that cluster. Every weight and adapter page links here ('you'll need a wrench').</t>
         </is>
@@ -2764,6 +2856,7 @@
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="6" t="n"/>
       <c r="M40" s="6" t="n"/>
+      <c r="N40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2802,7 +2895,8 @@
       <c r="J41" s="8" t="n"/>
       <c r="K41" s="8" t="n"/>
       <c r="L41" s="8" t="n"/>
-      <c r="M41" s="8" t="inlineStr">
+      <c r="M41" s="8" t="n"/>
+      <c r="N41" s="8" t="inlineStr">
         <is>
           <t>Keep this page plain — NO keyword-targeted copy or headings. It must not compete with the SEO pages.</t>
         </is>
@@ -2845,7 +2939,8 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="8" t="n"/>
-      <c r="M42" s="8" t="inlineStr">
+      <c r="M42" s="8" t="n"/>
+      <c r="N42" s="8" t="inlineStr">
         <is>
           <t>Keep this page plain — NO keyword-targeted copy or headings. It must not compete with the SEO pages.</t>
         </is>
@@ -2888,7 +2983,8 @@
       <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="n"/>
       <c r="L43" s="8" t="n"/>
-      <c r="M43" s="8" t="inlineStr">
+      <c r="M43" s="8" t="n"/>
+      <c r="N43" s="8" t="inlineStr">
         <is>
           <t>Keep this page plain — NO keyword-targeted copy or headings. It must not compete with the SEO pages.</t>
         </is>
@@ -2912,6 +3008,7 @@
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="6" t="n"/>
       <c r="M44" s="6" t="n"/>
+      <c r="N44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2966,7 +3063,8 @@
       </c>
       <c r="K45" s="8" t="n"/>
       <c r="L45" s="8" t="n"/>
-      <c r="M45" s="8" t="inlineStr">
+      <c r="M45" s="8" t="n"/>
+      <c r="N45" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Paradym Driver &amp; Fairway Wood') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -3025,7 +3123,8 @@
       </c>
       <c r="K46" s="8" t="n"/>
       <c r="L46" s="8" t="n"/>
-      <c r="M46" s="8" t="inlineStr">
+      <c r="M46" s="8" t="n"/>
+      <c r="N46" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Epic Speed &amp; Max Driver, Fairway &amp; Apex Utility Hybrid') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -3084,7 +3183,8 @@
       </c>
       <c r="K47" s="8" t="n"/>
       <c r="L47" s="8" t="n"/>
-      <c r="M47" s="8" t="inlineStr">
+      <c r="M47" s="8" t="n"/>
+      <c r="N47" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Mavrik, Sub Zero &amp; Max Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -3143,7 +3243,8 @@
       </c>
       <c r="K48" s="8" t="n"/>
       <c r="L48" s="8" t="n"/>
-      <c r="M48" s="8" t="inlineStr">
+      <c r="M48" s="8" t="n"/>
+      <c r="N48" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Epic Flash, Sub Zero &amp; Epic Max Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -3202,7 +3303,8 @@
       </c>
       <c r="K49" s="8" t="n"/>
       <c r="L49" s="8" t="n"/>
-      <c r="M49" s="8" t="inlineStr">
+      <c r="M49" s="8" t="n"/>
+      <c r="N49" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra Aerojet, Max &amp; LS Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -3261,7 +3363,8 @@
       </c>
       <c r="K50" s="8" t="n"/>
       <c r="L50" s="8" t="n"/>
-      <c r="M50" s="8" t="inlineStr">
+      <c r="M50" s="8" t="n"/>
+      <c r="N50" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra King Vintage Putter') — always include 'Weights'. Don't use the phrase 'Cobra putter weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -3320,7 +3423,8 @@
       </c>
       <c r="K51" s="8" t="n"/>
       <c r="L51" s="8" t="n"/>
-      <c r="M51" s="8" t="inlineStr">
+      <c r="M51" s="8" t="n"/>
+      <c r="N51" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra King Radspeed XB &amp; XD Driver') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -3379,7 +3483,8 @@
       </c>
       <c r="K52" s="8" t="n"/>
       <c r="L52" s="8" t="n"/>
-      <c r="M52" s="8" t="inlineStr">
+      <c r="M52" s="8" t="n"/>
+      <c r="N52" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra King Radspeed XB &amp; XD Driver Single Weight') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -3438,7 +3543,8 @@
       </c>
       <c r="K53" s="8" t="n"/>
       <c r="L53" s="8" t="n"/>
-      <c r="M53" s="8" t="inlineStr">
+      <c r="M53" s="8" t="n"/>
+      <c r="N53" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra SZ Speedzone Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -3497,7 +3603,8 @@
       </c>
       <c r="K54" s="8" t="n"/>
       <c r="L54" s="8" t="n"/>
-      <c r="M54" s="8" t="inlineStr">
+      <c r="M54" s="8" t="n"/>
+      <c r="N54" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Fastback &amp; Squareback Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -3556,7 +3663,8 @@
       </c>
       <c r="K55" s="8" t="n"/>
       <c r="L55" s="8" t="n"/>
-      <c r="M55" s="8" t="inlineStr">
+      <c r="M55" s="8" t="n"/>
+      <c r="N55" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Ai-ONE &amp; Ai-ONE Cruiser Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -3615,7 +3723,8 @@
       </c>
       <c r="K56" s="8" t="n"/>
       <c r="L56" s="8" t="n"/>
-      <c r="M56" s="8" t="inlineStr">
+      <c r="M56" s="8" t="n"/>
+      <c r="N56" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Stroke Lab, White Hot OG, Ten &amp; O-Works Putter Single Weights') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits. This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -3674,7 +3783,8 @@
       </c>
       <c r="K57" s="8" t="n"/>
       <c r="L57" s="8" t="n"/>
-      <c r="M57" s="8" t="inlineStr">
+      <c r="M57" s="8" t="n"/>
+      <c r="N57" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Stroke Lab &amp; White Hot Putter Single Weight') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -3733,7 +3843,8 @@
       </c>
       <c r="K58" s="8" t="n"/>
       <c r="L58" s="8" t="n"/>
-      <c r="M58" s="8" t="inlineStr">
+      <c r="M58" s="8" t="n"/>
+      <c r="N58" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G400 LST, SFT &amp; Max Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -3792,7 +3903,8 @@
       </c>
       <c r="K59" s="8" t="n"/>
       <c r="L59" s="8" t="n"/>
-      <c r="M59" s="8" t="inlineStr">
+      <c r="M59" s="8" t="n"/>
+      <c r="N59" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G410 Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -3851,7 +3963,8 @@
       </c>
       <c r="K60" s="8" t="n"/>
       <c r="L60" s="8" t="n"/>
-      <c r="M60" s="8" t="inlineStr">
+      <c r="M60" s="8" t="n"/>
+      <c r="N60" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G425 Fairway Wood &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping fairway wood weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -3910,7 +4023,8 @@
       </c>
       <c r="K61" s="8" t="n"/>
       <c r="L61" s="8" t="n"/>
-      <c r="M61" s="8" t="inlineStr">
+      <c r="M61" s="8" t="n"/>
+      <c r="N61" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G425 Driver Sliding') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -3969,7 +4083,8 @@
       </c>
       <c r="K62" s="8" t="n"/>
       <c r="L62" s="8" t="n"/>
-      <c r="M62" s="8" t="inlineStr">
+      <c r="M62" s="8" t="n"/>
+      <c r="N62" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Replacement Weights for Scotty Cameron Putters') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead). Also avoid 'putter weights' on its own — the Putter Head Weights collection owns that phrase.</t>
         </is>
@@ -4028,7 +4143,8 @@
       </c>
       <c r="K63" s="8" t="n"/>
       <c r="L63" s="8" t="n"/>
-      <c r="M63" s="8" t="inlineStr">
+      <c r="M63" s="8" t="n"/>
+      <c r="N63" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade SIM2, SIM2 Max &amp; Max D Driver Heel') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4087,7 +4203,8 @@
       </c>
       <c r="K64" s="8" t="n"/>
       <c r="L64" s="8" t="n"/>
-      <c r="M64" s="8" t="inlineStr">
+      <c r="M64" s="8" t="n"/>
+      <c r="N64" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade M5 Driver Sliding') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4146,7 +4263,8 @@
       </c>
       <c r="K65" s="8" t="n"/>
       <c r="L65" s="8" t="n"/>
-      <c r="M65" s="8" t="inlineStr">
+      <c r="M65" s="8" t="n"/>
+      <c r="N65" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade M2 Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4205,7 +4323,8 @@
       </c>
       <c r="K66" s="8" t="n"/>
       <c r="L66" s="8" t="n"/>
-      <c r="M66" s="8" t="inlineStr">
+      <c r="M66" s="8" t="n"/>
+      <c r="N66" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade BRNR Mini Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4264,7 +4383,8 @@
       </c>
       <c r="K67" s="8" t="n"/>
       <c r="L67" s="8" t="n"/>
-      <c r="M67" s="8" t="inlineStr">
+      <c r="M67" s="8" t="n"/>
+      <c r="N67" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade M1 Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4323,7 +4443,8 @@
       </c>
       <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="n"/>
-      <c r="M68" s="8" t="inlineStr">
+      <c r="M68" s="8" t="n"/>
+      <c r="N68" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade M2 D-Type Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4382,7 +4503,8 @@
       </c>
       <c r="K69" s="8" t="n"/>
       <c r="L69" s="8" t="n"/>
-      <c r="M69" s="8" t="inlineStr">
+      <c r="M69" s="8" t="n"/>
+      <c r="N69" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi10 Max, LS &amp; HL Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4441,7 +4563,8 @@
       </c>
       <c r="K70" s="8" t="n"/>
       <c r="L70" s="8" t="n"/>
-      <c r="M70" s="8" t="inlineStr">
+      <c r="M70" s="8" t="n"/>
+      <c r="N70" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade R7 Quad Mini Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4500,7 +4623,8 @@
       </c>
       <c r="K71" s="8" t="n"/>
       <c r="L71" s="8" t="n"/>
-      <c r="M71" s="8" t="inlineStr">
+      <c r="M71" s="8" t="n"/>
+      <c r="N71" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade TP Reserve &amp; Spider GTX Max Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4559,7 +4683,8 @@
       </c>
       <c r="K72" s="8" t="n"/>
       <c r="L72" s="8" t="n"/>
-      <c r="M72" s="8" t="inlineStr">
+      <c r="M72" s="8" t="n"/>
+      <c r="N72" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Stealth, Stealth HD &amp; Stealth Plus') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -4618,7 +4743,8 @@
       </c>
       <c r="K73" s="8" t="n"/>
       <c r="L73" s="8" t="n"/>
-      <c r="M73" s="8" t="inlineStr">
+      <c r="M73" s="8" t="n"/>
+      <c r="N73" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Stealth 2 Plus Driver &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead). Two of your pages currently rank for 'Stealth 2 Plus' — this one keeps it; the Stealth 2 kit page must lead with 'Weight Kit'.</t>
         </is>
@@ -4677,7 +4803,8 @@
       </c>
       <c r="K74" s="8" t="n"/>
       <c r="L74" s="8" t="n"/>
-      <c r="M74" s="8" t="inlineStr">
+      <c r="M74" s="8" t="n"/>
+      <c r="N74" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist TS3 Driver Magnetic SureFit') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -4736,7 +4863,8 @@
       </c>
       <c r="K75" s="8" t="n"/>
       <c r="L75" s="8" t="n"/>
-      <c r="M75" s="8" t="inlineStr">
+      <c r="M75" s="8" t="n"/>
+      <c r="N75" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Elyte X, Max &amp; Fast Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -4795,7 +4923,8 @@
       </c>
       <c r="K76" s="8" t="n"/>
       <c r="L76" s="8" t="n"/>
-      <c r="M76" s="8" t="inlineStr">
+      <c r="M76" s="8" t="n"/>
+      <c r="N76" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Paradym Ai Smoke Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -4854,7 +4983,8 @@
       </c>
       <c r="K77" s="8" t="n"/>
       <c r="L77" s="8" t="n"/>
-      <c r="M77" s="8" t="inlineStr">
+      <c r="M77" s="8" t="n"/>
+      <c r="N77" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Paradym Ai Smoke Fairway Wood') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -4913,7 +5043,8 @@
       </c>
       <c r="K78" s="8" t="n"/>
       <c r="L78" s="8" t="n"/>
-      <c r="M78" s="8" t="inlineStr">
+      <c r="M78" s="8" t="n"/>
+      <c r="N78" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Quantum Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -4972,7 +5103,8 @@
       </c>
       <c r="K79" s="8" t="n"/>
       <c r="L79" s="8" t="n"/>
-      <c r="M79" s="8" t="inlineStr">
+      <c r="M79" s="8" t="n"/>
+      <c r="N79" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Quantum Hybrid') — always include 'Weights'. Don't use the phrase 'Callaway hybrid weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -5031,7 +5163,8 @@
       </c>
       <c r="K80" s="8" t="n"/>
       <c r="L80" s="8" t="n"/>
-      <c r="M80" s="8" t="inlineStr">
+      <c r="M80" s="8" t="n"/>
+      <c r="N80" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra Darkspeed LS, Max &amp; X Driver') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -5090,7 +5223,8 @@
       </c>
       <c r="K81" s="8" t="n"/>
       <c r="L81" s="8" t="n"/>
-      <c r="M81" s="8" t="inlineStr">
+      <c r="M81" s="8" t="n"/>
+      <c r="N81" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra DS-Adapt Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -5149,7 +5283,8 @@
       </c>
       <c r="K82" s="8" t="n"/>
       <c r="L82" s="8" t="n"/>
-      <c r="M82" s="8" t="inlineStr">
+      <c r="M82" s="8" t="n"/>
+      <c r="N82" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G440 Driver') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -5208,7 +5343,8 @@
       </c>
       <c r="K83" s="8" t="n"/>
       <c r="L83" s="8" t="n"/>
-      <c r="M83" s="8" t="inlineStr">
+      <c r="M83" s="8" t="n"/>
+      <c r="N83" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G440 Fairway Wood') — always include 'Weights'. Don't use the phrase 'Ping fairway wood weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -5267,7 +5403,8 @@
       </c>
       <c r="K84" s="8" t="n"/>
       <c r="L84" s="8" t="n"/>
-      <c r="M84" s="8" t="inlineStr">
+      <c r="M84" s="8" t="n"/>
+      <c r="N84" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Srixon ZXi, ZXi LS &amp; ZXi Max Driver') — always include 'Weights'. Don't use the phrase 'Srixon driver weights' in this page's title or headings — that phrase belongs to the Srixon collection page (link to it instead).</t>
         </is>
@@ -5326,7 +5463,8 @@
       </c>
       <c r="K85" s="8" t="n"/>
       <c r="L85" s="8" t="n"/>
-      <c r="M85" s="8" t="inlineStr">
+      <c r="M85" s="8" t="n"/>
+      <c r="N85" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GT2 &amp; GT4 Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -5385,7 +5523,8 @@
       </c>
       <c r="K86" s="8" t="n"/>
       <c r="L86" s="8" t="n"/>
-      <c r="M86" s="8" t="inlineStr">
+      <c r="M86" s="8" t="n"/>
+      <c r="N86" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GT2 &amp; GT4 Hybrid') — always include 'Weights'. Don't use the phrase 'Titleist hybrid weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -5444,7 +5583,8 @@
       </c>
       <c r="K87" s="8" t="n"/>
       <c r="L87" s="8" t="n"/>
-      <c r="M87" s="8" t="inlineStr">
+      <c r="M87" s="8" t="n"/>
+      <c r="N87" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GT3 Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -5503,7 +5643,8 @@
       </c>
       <c r="K88" s="8" t="n"/>
       <c r="L88" s="8" t="n"/>
-      <c r="M88" s="8" t="inlineStr">
+      <c r="M88" s="8" t="n"/>
+      <c r="N88" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GT3 Fairway') — always include 'Weights'. Don't use the phrase 'Titleist fairway wood weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -5562,7 +5703,8 @@
       </c>
       <c r="K89" s="8" t="n"/>
       <c r="L89" s="8" t="n"/>
-      <c r="M89" s="8" t="inlineStr">
+      <c r="M89" s="8" t="n"/>
+      <c r="N89" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Epic Flash &amp; Rogue ST Sub Zero Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -5621,7 +5763,8 @@
       </c>
       <c r="K90" s="8" t="n"/>
       <c r="L90" s="8" t="n"/>
-      <c r="M90" s="8" t="inlineStr">
+      <c r="M90" s="8" t="n"/>
+      <c r="N90" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Apex Utility Wood') — always include 'Weights'. Don't use the phrase 'Callaway golf weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -5680,7 +5823,8 @@
       </c>
       <c r="K91" s="8" t="n"/>
       <c r="L91" s="8" t="n"/>
-      <c r="M91" s="8" t="inlineStr">
+      <c r="M91" s="8" t="n"/>
+      <c r="N91" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Apex Utility Wood') — always include 'Weights'. Don't use the phrase 'Callaway golf weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -5739,7 +5883,8 @@
       </c>
       <c r="K92" s="8" t="n"/>
       <c r="L92" s="8" t="n"/>
-      <c r="M92" s="8" t="inlineStr">
+      <c r="M92" s="8" t="n"/>
+      <c r="N92" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Paradym X &amp; Triple Diamond Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -5798,7 +5943,8 @@
       </c>
       <c r="K93" s="8" t="n"/>
       <c r="L93" s="8" t="n"/>
-      <c r="M93" s="8" t="inlineStr">
+      <c r="M93" s="8" t="n"/>
+      <c r="N93" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Paradym X &amp; Triple Diamond Fairway Wood') — always include 'Weights'. Don't use the phrase 'Callaway fairway wood weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -5857,7 +6003,8 @@
       </c>
       <c r="K94" s="8" t="n"/>
       <c r="L94" s="8" t="n"/>
-      <c r="M94" s="8" t="inlineStr">
+      <c r="M94" s="8" t="n"/>
+      <c r="N94" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Paradym X &amp; Triple Diamond Hybrid') — always include 'Weights'. Don't use the phrase 'Callaway hybrid weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -5916,7 +6063,8 @@
       </c>
       <c r="K95" s="8" t="n"/>
       <c r="L95" s="8" t="n"/>
-      <c r="M95" s="8" t="inlineStr">
+      <c r="M95" s="8" t="n"/>
+      <c r="N95" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Apex Hybrid') — always include 'Weights'. Don't use the phrase 'Callaway hybrid weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -5975,7 +6123,8 @@
       </c>
       <c r="K96" s="8" t="n"/>
       <c r="L96" s="8" t="n"/>
-      <c r="M96" s="8" t="inlineStr">
+      <c r="M96" s="8" t="n"/>
+      <c r="N96" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Epic Max &amp; Max LS Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -6034,7 +6183,8 @@
       </c>
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="n"/>
-      <c r="M97" s="8" t="inlineStr">
+      <c r="M97" s="8" t="n"/>
+      <c r="N97" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Epic Sub Zero Fairway &amp; Alpha 815') — always include 'Weights'. Don't use the phrase 'Callaway fairway wood weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -6093,7 +6243,8 @@
       </c>
       <c r="K98" s="8" t="n"/>
       <c r="L98" s="8" t="n"/>
-      <c r="M98" s="8" t="inlineStr">
+      <c r="M98" s="8" t="n"/>
+      <c r="N98" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Big Bertha B21 &amp; Reva Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -6152,7 +6303,8 @@
       </c>
       <c r="K99" s="8" t="n"/>
       <c r="L99" s="8" t="n"/>
-      <c r="M99" s="8" t="inlineStr">
+      <c r="M99" s="8" t="n"/>
+      <c r="N99" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Great Big Bertha, Alpha &amp; XR16 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -6211,7 +6363,8 @@
       </c>
       <c r="K100" s="8" t="n"/>
       <c r="L100" s="8" t="n"/>
-      <c r="M100" s="8" t="inlineStr">
+      <c r="M100" s="8" t="n"/>
+      <c r="N100" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Rogue Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -6270,7 +6423,8 @@
       </c>
       <c r="K101" s="8" t="n"/>
       <c r="L101" s="8" t="n"/>
-      <c r="M101" s="8" t="inlineStr">
+      <c r="M101" s="8" t="n"/>
+      <c r="N101" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra LTDx Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -6329,7 +6483,8 @@
       </c>
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="n"/>
-      <c r="M102" s="8" t="inlineStr">
+      <c r="M102" s="8" t="n"/>
+      <c r="N102" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra LTDx Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra fairway wood weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -6388,7 +6543,8 @@
       </c>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="n"/>
-      <c r="M103" s="8" t="inlineStr">
+      <c r="M103" s="8" t="n"/>
+      <c r="N103" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra OPTM Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -6447,7 +6603,8 @@
       </c>
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="n"/>
-      <c r="M104" s="8" t="inlineStr">
+      <c r="M104" s="8" t="n"/>
+      <c r="N104" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra SZ Speedzone Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra fairway wood weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -6506,7 +6663,8 @@
       </c>
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="8" t="n"/>
-      <c r="M105" s="8" t="inlineStr">
+      <c r="M105" s="8" t="n"/>
+      <c r="N105" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Honma T//World TR20 &amp; GS Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Honma driver weights' in this page's title or headings — that phrase belongs to the Honma collection page (link to it instead).</t>
         </is>
@@ -6565,7 +6723,8 @@
       </c>
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="n"/>
-      <c r="M106" s="8" t="inlineStr">
+      <c r="M106" s="8" t="n"/>
+      <c r="N106" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'LAB Golf Putter') — always include 'Weights'. Don't use the phrase 'LAB Golf putter weights' in this page's title or headings — that phrase belongs to the LAB Golf collection page (link to it instead).</t>
         </is>
@@ -6624,7 +6783,8 @@
       </c>
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="n"/>
-      <c r="M107" s="8" t="inlineStr">
+      <c r="M107" s="8" t="n"/>
+      <c r="N107" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Mizuno ST Range Driver') — always include 'Weights'. Don't use the phrase 'Mizuno driver weights' in this page's title or headings — that phrase belongs to the Mizuno collection page (link to it instead).</t>
         </is>
@@ -6683,7 +6843,8 @@
       </c>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
-      <c r="M108" s="8" t="inlineStr">
+      <c r="M108" s="8" t="n"/>
+      <c r="N108" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Golf Lead Tape — Self-Adhesive Swing Weight Tape') — always include 'Weights'.</t>
         </is>
@@ -6742,7 +6903,8 @@
       </c>
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="n"/>
-      <c r="M109" s="8" t="inlineStr">
+      <c r="M109" s="8" t="n"/>
+      <c r="N109" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Ai Dual &amp; Square 2 Square Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -6801,7 +6963,8 @@
       </c>
       <c r="K110" s="8" t="n"/>
       <c r="L110" s="8" t="n"/>
-      <c r="M110" s="8" t="inlineStr">
+      <c r="M110" s="8" t="n"/>
+      <c r="N110" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Ai-ONE Milled &amp; Toulon Ai Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -6860,7 +7023,8 @@
       </c>
       <c r="K111" s="8" t="n"/>
       <c r="L111" s="8" t="n"/>
-      <c r="M111" s="8" t="inlineStr">
+      <c r="M111" s="8" t="n"/>
+      <c r="N111" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Toulon 2022 Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -6919,7 +7083,8 @@
       </c>
       <c r="K112" s="8" t="n"/>
       <c r="L112" s="8" t="n"/>
-      <c r="M112" s="8" t="inlineStr">
+      <c r="M112" s="8" t="n"/>
+      <c r="N112" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Toulon 2025 Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -6978,7 +7143,8 @@
       </c>
       <c r="K113" s="8" t="n"/>
       <c r="L113" s="8" t="n"/>
-      <c r="M113" s="8" t="inlineStr">
+      <c r="M113" s="8" t="n"/>
+      <c r="N113" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Tri-Hot &amp; Square 2 Square Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -7037,7 +7203,8 @@
       </c>
       <c r="K114" s="8" t="n"/>
       <c r="L114" s="8" t="n"/>
-      <c r="M114" s="8" t="inlineStr">
+      <c r="M114" s="8" t="n"/>
+      <c r="N114" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Tri-Hot 5K Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -7096,7 +7263,8 @@
       </c>
       <c r="K115" s="8" t="n"/>
       <c r="L115" s="8" t="n"/>
-      <c r="M115" s="8" t="inlineStr">
+      <c r="M115" s="8" t="n"/>
+      <c r="N115" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'PXG Gen 8 Irons') — always include 'Weights'. Don't use the phrase 'PXG iron weights' in this page's title or headings — that phrase belongs to the PXG collection page (link to it instead).</t>
         </is>
@@ -7155,7 +7323,8 @@
       </c>
       <c r="K116" s="8" t="n"/>
       <c r="L116" s="8" t="n"/>
-      <c r="M116" s="8" t="inlineStr">
+      <c r="M116" s="8" t="n"/>
+      <c r="N116" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'PXG Gen 4 &amp; Gen 5 Irons') — always include 'Weights'. Don't use the phrase 'PXG iron weights' in this page's title or headings — that phrase belongs to the PXG collection page (link to it instead).</t>
         </is>
@@ -7214,7 +7383,8 @@
       </c>
       <c r="K117" s="8" t="n"/>
       <c r="L117" s="8" t="n"/>
-      <c r="M117" s="8" t="inlineStr">
+      <c r="M117" s="8" t="n"/>
+      <c r="N117" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'PXG Battle Ready Gen 2 Putter Single Weight') — always include 'Weights'. Don't use the phrase 'PXG putter weights' in this page's title or headings — that phrase belongs to the PXG collection page (link to it instead).</t>
         </is>
@@ -7273,7 +7443,8 @@
       </c>
       <c r="K118" s="8" t="n"/>
       <c r="L118" s="8" t="n"/>
-      <c r="M118" s="8" t="inlineStr">
+      <c r="M118" s="8" t="n"/>
+      <c r="N118" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'PXG Gen 4 0811, 0341 &amp; XGen 4 0211 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'PXG driver weights' in this page's title or headings — that phrase belongs to the PXG collection page (link to it instead).</t>
         </is>
@@ -7332,7 +7503,8 @@
       </c>
       <c r="K119" s="8" t="n"/>
       <c r="L119" s="8" t="n"/>
-      <c r="M119" s="8" t="inlineStr">
+      <c r="M119" s="8" t="n"/>
+      <c r="N119" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G30 LS &amp; SF Tec Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -7391,7 +7563,8 @@
       </c>
       <c r="K120" s="8" t="n"/>
       <c r="L120" s="8" t="n"/>
-      <c r="M120" s="8" t="inlineStr">
+      <c r="M120" s="8" t="n"/>
+      <c r="N120" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G430 Driver') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -7450,7 +7623,8 @@
       </c>
       <c r="K121" s="8" t="n"/>
       <c r="L121" s="8" t="n"/>
-      <c r="M121" s="8" t="inlineStr">
+      <c r="M121" s="8" t="n"/>
+      <c r="N121" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G430 Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -7509,7 +7683,8 @@
       </c>
       <c r="K122" s="8" t="n"/>
       <c r="L122" s="8" t="n"/>
-      <c r="M122" s="8" t="inlineStr">
+      <c r="M122" s="8" t="n"/>
+      <c r="N122" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Replacement Weights for Ping Irons') — always include 'Weights'. Don't use the phrase 'Ping iron weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -7568,7 +7743,8 @@
       </c>
       <c r="K123" s="8" t="n"/>
       <c r="L123" s="8" t="n"/>
-      <c r="M123" s="8" t="inlineStr">
+      <c r="M123" s="8" t="n"/>
+      <c r="N123" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping Vault 2.0 &amp; Classic Putter') — always include 'Weights'. Don't use the phrase 'Ping putter weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -7627,7 +7803,8 @@
       </c>
       <c r="K124" s="8" t="n"/>
       <c r="L124" s="8" t="n"/>
-      <c r="M124" s="8" t="inlineStr">
+      <c r="M124" s="8" t="n"/>
+      <c r="N124" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Putter Weights &amp; Wrench') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -7686,7 +7863,8 @@
       </c>
       <c r="K125" s="8" t="n"/>
       <c r="L125" s="8" t="n"/>
-      <c r="M125" s="8" t="inlineStr">
+      <c r="M125" s="8" t="n"/>
+      <c r="N125" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Blue Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -7745,7 +7923,8 @@
       </c>
       <c r="K126" s="8" t="n"/>
       <c r="L126" s="8" t="n"/>
-      <c r="M126" s="8" t="inlineStr">
+      <c r="M126" s="8" t="n"/>
+      <c r="N126" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Captain America Blue Star Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -7804,7 +7983,8 @@
       </c>
       <c r="K127" s="8" t="n"/>
       <c r="L127" s="8" t="n"/>
-      <c r="M127" s="8" t="inlineStr">
+      <c r="M127" s="8" t="n"/>
+      <c r="N127" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Circle T Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -7863,7 +8043,8 @@
       </c>
       <c r="K128" s="8" t="n"/>
       <c r="L128" s="8" t="n"/>
-      <c r="M128" s="8" t="inlineStr">
+      <c r="M128" s="8" t="n"/>
+      <c r="N128" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Circle T Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -7922,7 +8103,8 @@
       </c>
       <c r="K129" s="8" t="n"/>
       <c r="L129" s="8" t="n"/>
-      <c r="M129" s="8" t="inlineStr">
+      <c r="M129" s="8" t="n"/>
+      <c r="N129" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Copper Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -7981,7 +8163,8 @@
       </c>
       <c r="K130" s="8" t="n"/>
       <c r="L130" s="8" t="n"/>
-      <c r="M130" s="8" t="inlineStr">
+      <c r="M130" s="8" t="n"/>
+      <c r="N130" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Four Leaf Clover Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -8040,7 +8223,8 @@
       </c>
       <c r="K131" s="8" t="n"/>
       <c r="L131" s="8" t="n"/>
-      <c r="M131" s="8" t="inlineStr">
+      <c r="M131" s="8" t="n"/>
+      <c r="N131" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Gold Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -8099,7 +8283,8 @@
       </c>
       <c r="K132" s="8" t="n"/>
       <c r="L132" s="8" t="n"/>
-      <c r="M132" s="8" t="inlineStr">
+      <c r="M132" s="8" t="n"/>
+      <c r="N132" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -8158,7 +8343,8 @@
       </c>
       <c r="K133" s="8" t="n"/>
       <c r="L133" s="8" t="n"/>
-      <c r="M133" s="8" t="inlineStr">
+      <c r="M133" s="8" t="n"/>
+      <c r="N133" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -8217,7 +8403,8 @@
       </c>
       <c r="K134" s="8" t="n"/>
       <c r="L134" s="8" t="n"/>
-      <c r="M134" s="8" t="inlineStr">
+      <c r="M134" s="8" t="n"/>
+      <c r="N134" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Red Insert Fastback &amp; Squareback Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -8276,7 +8463,8 @@
       </c>
       <c r="K135" s="8" t="n"/>
       <c r="L135" s="8" t="n"/>
-      <c r="M135" s="8" t="inlineStr">
+      <c r="M135" s="8" t="n"/>
+      <c r="N135" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Red Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -8335,7 +8523,8 @@
       </c>
       <c r="K136" s="8" t="n"/>
       <c r="L136" s="8" t="n"/>
-      <c r="M136" s="8" t="inlineStr">
+      <c r="M136" s="8" t="n"/>
+      <c r="N136" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Rose Gold Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -8394,7 +8583,8 @@
       </c>
       <c r="K137" s="8" t="n"/>
       <c r="L137" s="8" t="n"/>
-      <c r="M137" s="8" t="inlineStr">
+      <c r="M137" s="8" t="n"/>
+      <c r="N137" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Superman Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -8453,7 +8643,8 @@
       </c>
       <c r="K138" s="8" t="n"/>
       <c r="L138" s="8" t="n"/>
-      <c r="M138" s="8" t="inlineStr">
+      <c r="M138" s="8" t="n"/>
+      <c r="N138" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Srixon ZX') — always include 'Weights'. Don't use the phrase 'Srixon golf weights' in this page's title or headings — that phrase belongs to the Srixon collection page (link to it instead).</t>
         </is>
@@ -8512,7 +8703,8 @@
       </c>
       <c r="K139" s="8" t="n"/>
       <c r="L139" s="8" t="n"/>
-      <c r="M139" s="8" t="inlineStr">
+      <c r="M139" s="8" t="n"/>
+      <c r="N139" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade TP Collection, Spider Mini, FSG &amp; Truss Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8571,7 +8763,8 @@
       </c>
       <c r="K140" s="8" t="n"/>
       <c r="L140" s="8" t="n"/>
-      <c r="M140" s="8" t="inlineStr">
+      <c r="M140" s="8" t="n"/>
+      <c r="N140" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade M3 Driver Sliding') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8630,7 +8823,8 @@
       </c>
       <c r="K141" s="8" t="n"/>
       <c r="L141" s="8" t="n"/>
-      <c r="M141" s="8" t="inlineStr">
+      <c r="M141" s="8" t="n"/>
+      <c r="N141" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi35 Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade golf weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8689,7 +8883,8 @@
       </c>
       <c r="K142" s="8" t="n"/>
       <c r="L142" s="8" t="n"/>
-      <c r="M142" s="8" t="inlineStr">
+      <c r="M142" s="8" t="n"/>
+      <c r="N142" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi35 Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'TaylorMade fairway wood weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8748,7 +8943,8 @@
       </c>
       <c r="K143" s="8" t="n"/>
       <c r="L143" s="8" t="n"/>
-      <c r="M143" s="8" t="inlineStr">
+      <c r="M143" s="8" t="n"/>
+      <c r="N143" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi4D Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade golf weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8807,7 +9003,8 @@
       </c>
       <c r="K144" s="8" t="n"/>
       <c r="L144" s="8" t="n"/>
-      <c r="M144" s="8" t="inlineStr">
+      <c r="M144" s="8" t="n"/>
+      <c r="N144" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade SIM Driver Back-Slider') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8866,7 +9063,8 @@
       </c>
       <c r="K145" s="8" t="n"/>
       <c r="L145" s="8" t="n"/>
-      <c r="M145" s="8" t="inlineStr">
+      <c r="M145" s="8" t="n"/>
+      <c r="N145" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade SIM Max D Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8925,7 +9123,8 @@
       </c>
       <c r="K146" s="8" t="n"/>
       <c r="L146" s="8" t="n"/>
-      <c r="M146" s="8" t="inlineStr">
+      <c r="M146" s="8" t="n"/>
+      <c r="N146" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade SIM Max Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -8984,7 +9183,8 @@
       </c>
       <c r="K147" s="8" t="n"/>
       <c r="L147" s="8" t="n"/>
-      <c r="M147" s="8" t="inlineStr">
+      <c r="M147" s="8" t="n"/>
+      <c r="N147" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Spider Tour Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9043,7 +9243,8 @@
       </c>
       <c r="K148" s="8" t="n"/>
       <c r="L148" s="8" t="n"/>
-      <c r="M148" s="8" t="inlineStr">
+      <c r="M148" s="8" t="n"/>
+      <c r="N148" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade TP Hydroblast &amp; Truss Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9102,7 +9303,8 @@
       </c>
       <c r="K149" s="8" t="n"/>
       <c r="L149" s="8" t="n"/>
-      <c r="M149" s="8" t="inlineStr">
+      <c r="M149" s="8" t="n"/>
+      <c r="N149" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Spider EX Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9161,7 +9363,8 @@
       </c>
       <c r="K150" s="8" t="n"/>
       <c r="L150" s="8" t="n"/>
-      <c r="M150" s="8" t="inlineStr">
+      <c r="M150" s="8" t="n"/>
+      <c r="N150" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade M4 Driver &amp; M4 Tour Fairway') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9220,7 +9423,8 @@
       </c>
       <c r="K151" s="8" t="n"/>
       <c r="L151" s="8" t="n"/>
-      <c r="M151" s="8" t="inlineStr">
+      <c r="M151" s="8" t="n"/>
+      <c r="N151" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade M6 Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9279,7 +9483,8 @@
       </c>
       <c r="K152" s="8" t="n"/>
       <c r="L152" s="8" t="n"/>
-      <c r="M152" s="8" t="inlineStr">
+      <c r="M152" s="8" t="n"/>
+      <c r="N152" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade R1, R5, R7, R9 &amp; R11 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9338,7 +9543,8 @@
       </c>
       <c r="K153" s="8" t="n"/>
       <c r="L153" s="8" t="n"/>
-      <c r="M153" s="8" t="inlineStr">
+      <c r="M153" s="8" t="n"/>
+      <c r="N153" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade SIM Titanium Fairway &amp; SIM UDI Utility Iron') — always include 'Weights'. Don't use the phrase 'TaylorMade fairway wood weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9397,7 +9603,8 @@
       </c>
       <c r="K154" s="8" t="n"/>
       <c r="L154" s="8" t="n"/>
-      <c r="M154" s="8" t="inlineStr">
+      <c r="M154" s="8" t="n"/>
+      <c r="N154" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Spider X &amp; MySpider X Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9456,7 +9663,8 @@
       </c>
       <c r="K155" s="8" t="n"/>
       <c r="L155" s="8" t="n"/>
-      <c r="M155" s="8" t="inlineStr">
+      <c r="M155" s="8" t="n"/>
+      <c r="N155" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Spider Tour Putter Single Weight') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -9515,7 +9723,8 @@
       </c>
       <c r="K156" s="8" t="n"/>
       <c r="L156" s="8" t="n"/>
-      <c r="M156" s="8" t="inlineStr">
+      <c r="M156" s="8" t="n"/>
+      <c r="N156" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist TSi2 &amp; TSi4 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -9574,7 +9783,8 @@
       </c>
       <c r="K157" s="8" t="n"/>
       <c r="L157" s="8" t="n"/>
-      <c r="M157" s="8" t="inlineStr">
+      <c r="M157" s="8" t="n"/>
+      <c r="N157" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist TS2 &amp; TS4 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -9633,7 +9843,8 @@
       </c>
       <c r="K158" s="8" t="n"/>
       <c r="L158" s="8" t="n"/>
-      <c r="M158" s="8" t="inlineStr">
+      <c r="M158" s="8" t="n"/>
+      <c r="N158" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist TSi2 &amp; TSi4 Driver &amp; Fairway Single Weight') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -9692,7 +9903,8 @@
       </c>
       <c r="K159" s="8" t="n"/>
       <c r="L159" s="8" t="n"/>
-      <c r="M159" s="8" t="inlineStr">
+      <c r="M159" s="8" t="n"/>
+      <c r="N159" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GTS2, GTS3 &amp; GTS4 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -9751,7 +9963,8 @@
       </c>
       <c r="K160" s="8" t="n"/>
       <c r="L160" s="8" t="n"/>
-      <c r="M160" s="8" t="inlineStr">
+      <c r="M160" s="8" t="n"/>
+      <c r="N160" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist TSi3 Driver') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -9810,7 +10023,8 @@
       </c>
       <c r="K161" s="8" t="n"/>
       <c r="L161" s="8" t="n"/>
-      <c r="M161" s="8" t="inlineStr">
+      <c r="M161" s="8" t="n"/>
+      <c r="N161" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist TS1 Driver Head Screw') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -9834,6 +10048,7 @@
       <c r="K162" s="6" t="n"/>
       <c r="L162" s="6" t="n"/>
       <c r="M162" s="6" t="n"/>
+      <c r="N162" s="6" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -9884,7 +10099,8 @@
       <c r="J163" s="8" t="n"/>
       <c r="K163" s="8" t="n"/>
       <c r="L163" s="8" t="n"/>
-      <c r="M163" s="8" t="inlineStr">
+      <c r="M163" s="8" t="n"/>
+      <c r="N163" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Mavrik, Sub Zero &amp; Max Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -9939,7 +10155,8 @@
       <c r="J164" s="8" t="n"/>
       <c r="K164" s="8" t="n"/>
       <c r="L164" s="8" t="n"/>
-      <c r="M164" s="8" t="inlineStr">
+      <c r="M164" s="8" t="n"/>
+      <c r="N164" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra Aerojet, Max &amp; LS Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -9994,7 +10211,8 @@
       <c r="J165" s="8" t="n"/>
       <c r="K165" s="8" t="n"/>
       <c r="L165" s="8" t="n"/>
-      <c r="M165" s="8" t="inlineStr">
+      <c r="M165" s="8" t="n"/>
+      <c r="N165" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Black, Stroke Lab, White Hot OG, Ten &amp; O-Works Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -10049,7 +10267,8 @@
       <c r="J166" s="8" t="n"/>
       <c r="K166" s="8" t="n"/>
       <c r="L166" s="8" t="n"/>
-      <c r="M166" s="8" t="inlineStr">
+      <c r="M166" s="8" t="n"/>
+      <c r="N166" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Stroke Lab, White Hot OG, Ten &amp; O-Works Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -10104,7 +10323,8 @@
       <c r="J167" s="8" t="n"/>
       <c r="K167" s="8" t="n"/>
       <c r="L167" s="8" t="n"/>
-      <c r="M167" s="8" t="inlineStr">
+      <c r="M167" s="8" t="n"/>
+      <c r="N167" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi10 Max, LS &amp; HL Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -10159,7 +10379,8 @@
       <c r="J168" s="8" t="n"/>
       <c r="K168" s="8" t="n"/>
       <c r="L168" s="8" t="n"/>
-      <c r="M168" s="8" t="inlineStr">
+      <c r="M168" s="8" t="n"/>
+      <c r="N168" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade R7 Quad Mini Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -10214,7 +10435,8 @@
       <c r="J169" s="8" t="n"/>
       <c r="K169" s="8" t="n"/>
       <c r="L169" s="8" t="n"/>
-      <c r="M169" s="8" t="inlineStr">
+      <c r="M169" s="8" t="n"/>
+      <c r="N169" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Elyte X, Max &amp; Fast Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -10269,7 +10491,8 @@
       <c r="J170" s="8" t="n"/>
       <c r="K170" s="8" t="n"/>
       <c r="L170" s="8" t="n"/>
-      <c r="M170" s="8" t="inlineStr">
+      <c r="M170" s="8" t="n"/>
+      <c r="N170" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Quantum Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -10324,7 +10547,8 @@
       <c r="J171" s="8" t="n"/>
       <c r="K171" s="8" t="n"/>
       <c r="L171" s="8" t="n"/>
-      <c r="M171" s="8" t="inlineStr">
+      <c r="M171" s="8" t="n"/>
+      <c r="N171" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra Darkspeed LS, Max &amp; X Driver') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -10379,7 +10603,8 @@
       <c r="J172" s="8" t="n"/>
       <c r="K172" s="8" t="n"/>
       <c r="L172" s="8" t="n"/>
-      <c r="M172" s="8" t="inlineStr">
+      <c r="M172" s="8" t="n"/>
+      <c r="N172" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra DS-Adapt Driver') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -10434,7 +10659,8 @@
       <c r="J173" s="8" t="n"/>
       <c r="K173" s="8" t="n"/>
       <c r="L173" s="8" t="n"/>
-      <c r="M173" s="8" t="inlineStr">
+      <c r="M173" s="8" t="n"/>
+      <c r="N173" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra DS-Adapt Fairway') — always include 'Weights'. Don't use the phrase 'Cobra fairway wood weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -10489,7 +10715,8 @@
       <c r="J174" s="8" t="n"/>
       <c r="K174" s="8" t="n"/>
       <c r="L174" s="8" t="n"/>
-      <c r="M174" s="8" t="inlineStr">
+      <c r="M174" s="8" t="n"/>
+      <c r="N174" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'PXG Black Ops, Gen 4–6') — always include 'Weights'. Don't use the phrase 'PXG driver weights' in this page's title or headings — that phrase belongs to the PXG collection page (link to it instead).</t>
         </is>
@@ -10544,7 +10771,8 @@
       <c r="J175" s="8" t="n"/>
       <c r="K175" s="8" t="n"/>
       <c r="L175" s="8" t="n"/>
-      <c r="M175" s="8" t="inlineStr">
+      <c r="M175" s="8" t="n"/>
+      <c r="N175" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G440 Driver') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -10599,7 +10827,8 @@
       <c r="J176" s="8" t="n"/>
       <c r="K176" s="8" t="n"/>
       <c r="L176" s="8" t="n"/>
-      <c r="M176" s="8" t="inlineStr">
+      <c r="M176" s="8" t="n"/>
+      <c r="N176" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G440 Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping fairway wood weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -10654,7 +10883,8 @@
       <c r="J177" s="8" t="n"/>
       <c r="K177" s="8" t="n"/>
       <c r="L177" s="8" t="n"/>
-      <c r="M177" s="8" t="inlineStr">
+      <c r="M177" s="8" t="n"/>
+      <c r="N177" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Srixon ZXi, ZXi LS &amp; ZXi Max Driver') — always include 'Weights'. Don't use the phrase 'Srixon driver weights' in this page's title or headings — that phrase belongs to the Srixon collection page (link to it instead).</t>
         </is>
@@ -10709,7 +10939,8 @@
       <c r="J178" s="8" t="n"/>
       <c r="K178" s="8" t="n"/>
       <c r="L178" s="8" t="n"/>
-      <c r="M178" s="8" t="inlineStr">
+      <c r="M178" s="8" t="n"/>
+      <c r="N178" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GT2 &amp; GT4 Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -10764,7 +10995,8 @@
       <c r="J179" s="8" t="n"/>
       <c r="K179" s="8" t="n"/>
       <c r="L179" s="8" t="n"/>
-      <c r="M179" s="8" t="inlineStr">
+      <c r="M179" s="8" t="n"/>
+      <c r="N179" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GT3 Driver') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -10819,7 +11051,8 @@
       <c r="J180" s="8" t="n"/>
       <c r="K180" s="8" t="n"/>
       <c r="L180" s="8" t="n"/>
-      <c r="M180" s="8" t="inlineStr">
+      <c r="M180" s="8" t="n"/>
+      <c r="N180" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Big Bertha B21 &amp; Reva Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -10874,7 +11107,8 @@
       <c r="J181" s="8" t="n"/>
       <c r="K181" s="8" t="n"/>
       <c r="L181" s="8" t="n"/>
-      <c r="M181" s="8" t="inlineStr">
+      <c r="M181" s="8" t="n"/>
+      <c r="N181" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Epic Speed Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -10929,7 +11163,8 @@
       <c r="J182" s="8" t="n"/>
       <c r="K182" s="8" t="n"/>
       <c r="L182" s="8" t="n"/>
-      <c r="M182" s="8" t="inlineStr">
+      <c r="M182" s="8" t="n"/>
+      <c r="N182" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Great Big Bertha, Alpha &amp; XR16 Driver') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -10984,7 +11219,8 @@
       <c r="J183" s="8" t="n"/>
       <c r="K183" s="8" t="n"/>
       <c r="L183" s="8" t="n"/>
-      <c r="M183" s="8" t="inlineStr">
+      <c r="M183" s="8" t="n"/>
+      <c r="N183" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Callaway Rogue Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Callaway driver weights' in this page's title or headings — that phrase belongs to the Callaway collection page (link to it instead).</t>
         </is>
@@ -11039,7 +11275,8 @@
       <c r="J184" s="8" t="n"/>
       <c r="K184" s="8" t="n"/>
       <c r="L184" s="8" t="n"/>
-      <c r="M184" s="8" t="inlineStr">
+      <c r="M184" s="8" t="n"/>
+      <c r="N184" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra King Radspeed XB &amp; XD Driver') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -11094,7 +11331,8 @@
       <c r="J185" s="8" t="n"/>
       <c r="K185" s="8" t="n"/>
       <c r="L185" s="8" t="n"/>
-      <c r="M185" s="8" t="inlineStr">
+      <c r="M185" s="8" t="n"/>
+      <c r="N185" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra King Vintage 3D Printed Putter') — always include 'Weights'. Don't use the phrase 'Cobra putter weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -11149,7 +11387,8 @@
       <c r="J186" s="8" t="n"/>
       <c r="K186" s="8" t="n"/>
       <c r="L186" s="8" t="n"/>
-      <c r="M186" s="8" t="inlineStr">
+      <c r="M186" s="8" t="n"/>
+      <c r="N186" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra LTDx Driver') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -11204,7 +11443,8 @@
       <c r="J187" s="8" t="n"/>
       <c r="K187" s="8" t="n"/>
       <c r="L187" s="8" t="n"/>
-      <c r="M187" s="8" t="inlineStr">
+      <c r="M187" s="8" t="n"/>
+      <c r="N187" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Cobra OPTM Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Cobra driver weights' in this page's title or headings — that phrase belongs to the Cobra collection page (link to it instead).</t>
         </is>
@@ -11259,7 +11499,8 @@
       <c r="J188" s="8" t="n"/>
       <c r="K188" s="8" t="n"/>
       <c r="L188" s="8" t="n"/>
-      <c r="M188" s="8" t="inlineStr">
+      <c r="M188" s="8" t="n"/>
+      <c r="N188" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Ai-ONE &amp; Ai-ONE Cruiser Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -11314,7 +11555,8 @@
       <c r="J189" s="8" t="n"/>
       <c r="K189" s="8" t="n"/>
       <c r="L189" s="8" t="n"/>
-      <c r="M189" s="8" t="inlineStr">
+      <c r="M189" s="8" t="n"/>
+      <c r="N189" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Ai-ONE Milled &amp; Toulon Ai Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -11369,7 +11611,8 @@
       <c r="J190" s="8" t="n"/>
       <c r="K190" s="8" t="n"/>
       <c r="L190" s="8" t="n"/>
-      <c r="M190" s="8" t="inlineStr">
+      <c r="M190" s="8" t="n"/>
+      <c r="N190" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Toulon 2025 Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -11424,7 +11667,8 @@
       <c r="J191" s="8" t="n"/>
       <c r="K191" s="8" t="n"/>
       <c r="L191" s="8" t="n"/>
-      <c r="M191" s="8" t="inlineStr">
+      <c r="M191" s="8" t="n"/>
+      <c r="N191" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Odyssey Tri-Hot 5K, Eleven, White Hot &amp; Versa Putter') — always include 'Weights'. Don't use the phrase 'Odyssey putter weights' in this page's title or headings — that phrase belongs to the Odyssey collection page (link to it instead). Three pages currently compete for 'Odyssey putter weights' — keep this page strictly about the models it fits.</t>
         </is>
@@ -11479,7 +11723,8 @@
       <c r="J192" s="8" t="n"/>
       <c r="K192" s="8" t="n"/>
       <c r="L192" s="8" t="n"/>
-      <c r="M192" s="8" t="inlineStr">
+      <c r="M192" s="8" t="n"/>
+      <c r="N192" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'PXG Battle Ready &amp; Battle Ready II Putter') — always include 'Weights'. Don't use the phrase 'PXG putter weights' in this page's title or headings — that phrase belongs to the PXG collection page (link to it instead).</t>
         </is>
@@ -11534,7 +11779,8 @@
       <c r="J193" s="8" t="n"/>
       <c r="K193" s="8" t="n"/>
       <c r="L193" s="8" t="n"/>
-      <c r="M193" s="8" t="inlineStr">
+      <c r="M193" s="8" t="n"/>
+      <c r="N193" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G425 Max &amp; LST Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping fairway wood weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -11589,7 +11835,8 @@
       <c r="J194" s="8" t="n"/>
       <c r="K194" s="8" t="n"/>
       <c r="L194" s="8" t="n"/>
-      <c r="M194" s="8" t="inlineStr">
+      <c r="M194" s="8" t="n"/>
+      <c r="N194" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G425 Max, LST &amp; SFT Driver') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -11644,7 +11891,8 @@
       <c r="J195" s="8" t="n"/>
       <c r="K195" s="8" t="n"/>
       <c r="L195" s="8" t="n"/>
-      <c r="M195" s="8" t="inlineStr">
+      <c r="M195" s="8" t="n"/>
+      <c r="N195" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G430 Driver') — always include 'Weights'. Don't use the phrase 'Ping driver weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -11699,7 +11947,8 @@
       <c r="J196" s="8" t="n"/>
       <c r="K196" s="8" t="n"/>
       <c r="L196" s="8" t="n"/>
-      <c r="M196" s="8" t="inlineStr">
+      <c r="M196" s="8" t="n"/>
+      <c r="N196" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Ping G430 Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'Ping fairway wood weights' in this page's title or headings — that phrase belongs to the Ping collection page (link to it instead).</t>
         </is>
@@ -11754,7 +12003,8 @@
       <c r="J197" s="8" t="n"/>
       <c r="K197" s="8" t="n"/>
       <c r="L197" s="8" t="n"/>
-      <c r="M197" s="8" t="inlineStr">
+      <c r="M197" s="8" t="n"/>
+      <c r="N197" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Black Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -11809,7 +12059,8 @@
       <c r="J198" s="8" t="n"/>
       <c r="K198" s="8" t="n"/>
       <c r="L198" s="8" t="n"/>
-      <c r="M198" s="8" t="inlineStr">
+      <c r="M198" s="8" t="n"/>
+      <c r="N198" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Blue Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -11864,7 +12115,8 @@
       <c r="J199" s="8" t="n"/>
       <c r="K199" s="8" t="n"/>
       <c r="L199" s="8" t="n"/>
-      <c r="M199" s="8" t="inlineStr">
+      <c r="M199" s="8" t="n"/>
+      <c r="N199" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Captain America Blue Star Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -11919,7 +12171,8 @@
       <c r="J200" s="8" t="n"/>
       <c r="K200" s="8" t="n"/>
       <c r="L200" s="8" t="n"/>
-      <c r="M200" s="8" t="inlineStr">
+      <c r="M200" s="8" t="n"/>
+      <c r="N200" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Circle T Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -11974,7 +12227,8 @@
       <c r="J201" s="8" t="n"/>
       <c r="K201" s="8" t="n"/>
       <c r="L201" s="8" t="n"/>
-      <c r="M201" s="8" t="inlineStr">
+      <c r="M201" s="8" t="n"/>
+      <c r="N201" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Circle T Red Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12029,7 +12283,8 @@
       <c r="J202" s="8" t="n"/>
       <c r="K202" s="8" t="n"/>
       <c r="L202" s="8" t="n"/>
-      <c r="M202" s="8" t="inlineStr">
+      <c r="M202" s="8" t="n"/>
+      <c r="N202" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Copper Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12084,7 +12339,8 @@
       <c r="J203" s="8" t="n"/>
       <c r="K203" s="8" t="n"/>
       <c r="L203" s="8" t="n"/>
-      <c r="M203" s="8" t="inlineStr">
+      <c r="M203" s="8" t="n"/>
+      <c r="N203" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Gold Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12139,7 +12395,8 @@
       <c r="J204" s="8" t="n"/>
       <c r="K204" s="8" t="n"/>
       <c r="L204" s="8" t="n"/>
-      <c r="M204" s="8" t="inlineStr">
+      <c r="M204" s="8" t="n"/>
+      <c r="N204" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Green Clover Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12194,7 +12451,8 @@
       <c r="J205" s="8" t="n"/>
       <c r="K205" s="8" t="n"/>
       <c r="L205" s="8" t="n"/>
-      <c r="M205" s="8" t="inlineStr">
+      <c r="M205" s="8" t="n"/>
+      <c r="N205" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12249,7 +12507,8 @@
       <c r="J206" s="8" t="n"/>
       <c r="K206" s="8" t="n"/>
       <c r="L206" s="8" t="n"/>
-      <c r="M206" s="8" t="inlineStr">
+      <c r="M206" s="8" t="n"/>
+      <c r="N206" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead). This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -12304,7 +12563,8 @@
       <c r="J207" s="8" t="n"/>
       <c r="K207" s="8" t="n"/>
       <c r="L207" s="8" t="n"/>
-      <c r="M207" s="8" t="inlineStr">
+      <c r="M207" s="8" t="n"/>
+      <c r="N207" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Putter Multi-Piece') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12359,7 +12619,8 @@
       <c r="J208" s="8" t="n"/>
       <c r="K208" s="8" t="n"/>
       <c r="L208" s="8" t="n"/>
-      <c r="M208" s="8" t="inlineStr">
+      <c r="M208" s="8" t="n"/>
+      <c r="N208" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Rose Gold Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12414,7 +12675,8 @@
       <c r="J209" s="8" t="n"/>
       <c r="K209" s="8" t="n"/>
       <c r="L209" s="8" t="n"/>
-      <c r="M209" s="8" t="inlineStr">
+      <c r="M209" s="8" t="n"/>
+      <c r="N209" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Scotty Cameron Superman Insert Putter') — always include 'Weights'. Don't use the phrase 'Scotty Cameron putter weights' in this page's title or headings — that phrase belongs to the Scotty Cameron collection page (link to it instead).</t>
         </is>
@@ -12469,7 +12731,8 @@
       <c r="J210" s="8" t="n"/>
       <c r="K210" s="8" t="n"/>
       <c r="L210" s="8" t="n"/>
-      <c r="M210" s="8" t="inlineStr">
+      <c r="M210" s="8" t="n"/>
+      <c r="N210" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Srixon ZX5 &amp; ZX7') — always include 'Weights'. Don't use the phrase 'Srixon driver weights' in this page's title or headings — that phrase belongs to the Srixon collection page (link to it instead).</t>
         </is>
@@ -12524,7 +12787,8 @@
       <c r="J211" s="8" t="n"/>
       <c r="K211" s="8" t="n"/>
       <c r="L211" s="8" t="n"/>
-      <c r="M211" s="8" t="inlineStr">
+      <c r="M211" s="8" t="n"/>
+      <c r="N211" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Burner Mini Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12579,7 +12843,8 @@
       <c r="J212" s="8" t="n"/>
       <c r="K212" s="8" t="n"/>
       <c r="L212" s="8" t="n"/>
-      <c r="M212" s="8" t="inlineStr">
+      <c r="M212" s="8" t="n"/>
+      <c r="N212" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade TP Collection, Spider Mini, FCG &amp; Truss Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12634,7 +12899,8 @@
       <c r="J213" s="8" t="n"/>
       <c r="K213" s="8" t="n"/>
       <c r="L213" s="8" t="n"/>
-      <c r="M213" s="8" t="inlineStr">
+      <c r="M213" s="8" t="n"/>
+      <c r="N213" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi35 Driver') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12689,7 +12955,8 @@
       <c r="J214" s="8" t="n"/>
       <c r="K214" s="8" t="n"/>
       <c r="L214" s="8" t="n"/>
-      <c r="M214" s="8" t="inlineStr">
+      <c r="M214" s="8" t="n"/>
+      <c r="N214" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi35 Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'TaylorMade fairway wood weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12744,7 +13011,8 @@
       <c r="J215" s="8" t="n"/>
       <c r="K215" s="8" t="n"/>
       <c r="L215" s="8" t="n"/>
-      <c r="M215" s="8" t="inlineStr">
+      <c r="M215" s="8" t="n"/>
+      <c r="N215" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Qi4D Driver, Fairway &amp; Hybrid') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12799,7 +13067,8 @@
       <c r="J216" s="8" t="n"/>
       <c r="K216" s="8" t="n"/>
       <c r="L216" s="8" t="n"/>
-      <c r="M216" s="8" t="inlineStr">
+      <c r="M216" s="8" t="n"/>
+      <c r="N216" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Spider Tour Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12854,7 +13123,8 @@
       <c r="J217" s="8" t="n"/>
       <c r="K217" s="8" t="n"/>
       <c r="L217" s="8" t="n"/>
-      <c r="M217" s="8" t="inlineStr">
+      <c r="M217" s="8" t="n"/>
+      <c r="N217" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade Stealth 2, Stealth 2 Plus &amp; Stealth 2 HD') — always include 'Weights'. Don't use the phrase 'TaylorMade driver weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12909,7 +13179,8 @@
       <c r="J218" s="8" t="n"/>
       <c r="K218" s="8" t="n"/>
       <c r="L218" s="8" t="n"/>
-      <c r="M218" s="8" t="inlineStr">
+      <c r="M218" s="8" t="n"/>
+      <c r="N218" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'TaylorMade TP Hydroblast &amp; Truss Putter') — always include 'Weights'. Don't use the phrase 'TaylorMade putter weights' in this page's title or headings — that phrase belongs to the TaylorMade collection page (link to it instead).</t>
         </is>
@@ -12964,7 +13235,8 @@
       <c r="J219" s="8" t="n"/>
       <c r="K219" s="8" t="n"/>
       <c r="L219" s="8" t="n"/>
-      <c r="M219" s="8" t="inlineStr">
+      <c r="M219" s="8" t="n"/>
+      <c r="N219" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist GTS2, GTS3 &amp; GTS4 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -13019,7 +13291,8 @@
       <c r="J220" s="8" t="n"/>
       <c r="K220" s="8" t="n"/>
       <c r="L220" s="8" t="n"/>
-      <c r="M220" s="8" t="inlineStr">
+      <c r="M220" s="8" t="n"/>
+      <c r="N220" s="8" t="inlineStr">
         <is>
           <t>Never use the bare club name on its own as the title (e.g. just 'Titleist TSR1, TSR2 &amp; TSR4 Driver &amp; Fairway') — always include 'Weights'. Don't use the phrase 'Titleist driver weights' in this page's title or headings — that phrase belongs to the Titleist collection page (link to it instead).</t>
         </is>
@@ -13043,6 +13316,7 @@
       <c r="K221" s="6" t="n"/>
       <c r="L221" s="6" t="n"/>
       <c r="M221" s="6" t="n"/>
+      <c r="N221" s="6" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="7" t="inlineStr">
@@ -13093,7 +13367,8 @@
       <c r="J222" s="8" t="n"/>
       <c r="K222" s="8" t="n"/>
       <c r="L222" s="8" t="n"/>
-      <c r="M222" s="8" t="inlineStr">
+      <c r="M222" s="8" t="n"/>
+      <c r="N222" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'TaylorMade shaft adapters' (plural) — that belongs to the TaylorMade adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13148,7 +13423,8 @@
       <c r="J223" s="8" t="n"/>
       <c r="K223" s="8" t="n"/>
       <c r="L223" s="8" t="n"/>
-      <c r="M223" s="8" t="inlineStr">
+      <c r="M223" s="8" t="n"/>
+      <c r="N223" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'TaylorMade shaft adapters' (plural) — that belongs to the TaylorMade adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13203,7 +13479,8 @@
       <c r="J224" s="8" t="n"/>
       <c r="K224" s="8" t="n"/>
       <c r="L224" s="8" t="n"/>
-      <c r="M224" s="8" t="inlineStr">
+      <c r="M224" s="8" t="n"/>
+      <c r="N224" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Titleist shaft adapters' (plural) — that belongs to the Titleist adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13258,7 +13535,8 @@
       <c r="J225" s="8" t="n"/>
       <c r="K225" s="8" t="n"/>
       <c r="L225" s="8" t="n"/>
-      <c r="M225" s="8" t="inlineStr">
+      <c r="M225" s="8" t="n"/>
+      <c r="N225" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Callaway shaft adapters' (plural) — that belongs to the Callaway adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13313,7 +13591,8 @@
       <c r="J226" s="8" t="n"/>
       <c r="K226" s="8" t="n"/>
       <c r="L226" s="8" t="n"/>
-      <c r="M226" s="8" t="inlineStr">
+      <c r="M226" s="8" t="n"/>
+      <c r="N226" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Callaway shaft adapters' (plural) — that belongs to the Callaway adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13368,7 +13647,8 @@
       <c r="J227" s="8" t="n"/>
       <c r="K227" s="8" t="n"/>
       <c r="L227" s="8" t="n"/>
-      <c r="M227" s="8" t="inlineStr">
+      <c r="M227" s="8" t="n"/>
+      <c r="N227" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Callaway shaft adapters' (plural) — that belongs to the Callaway adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13423,7 +13703,8 @@
       <c r="J228" s="8" t="n"/>
       <c r="K228" s="8" t="n"/>
       <c r="L228" s="8" t="n"/>
-      <c r="M228" s="8" t="inlineStr">
+      <c r="M228" s="8" t="n"/>
+      <c r="N228" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13478,7 +13759,8 @@
       <c r="J229" s="8" t="n"/>
       <c r="K229" s="8" t="n"/>
       <c r="L229" s="8" t="n"/>
-      <c r="M229" s="8" t="inlineStr">
+      <c r="M229" s="8" t="n"/>
+      <c r="N229" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13533,7 +13815,8 @@
       <c r="J230" s="8" t="n"/>
       <c r="K230" s="8" t="n"/>
       <c r="L230" s="8" t="n"/>
-      <c r="M230" s="8" t="inlineStr">
+      <c r="M230" s="8" t="n"/>
+      <c r="N230" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13588,7 +13871,8 @@
       <c r="J231" s="8" t="n"/>
       <c r="K231" s="8" t="n"/>
       <c r="L231" s="8" t="n"/>
-      <c r="M231" s="8" t="inlineStr">
+      <c r="M231" s="8" t="n"/>
+      <c r="N231" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13643,7 +13927,8 @@
       <c r="J232" s="8" t="n"/>
       <c r="K232" s="8" t="n"/>
       <c r="L232" s="8" t="n"/>
-      <c r="M232" s="8" t="inlineStr">
+      <c r="M232" s="8" t="n"/>
+      <c r="N232" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13698,7 +13983,8 @@
       <c r="J233" s="8" t="n"/>
       <c r="K233" s="8" t="n"/>
       <c r="L233" s="8" t="n"/>
-      <c r="M233" s="8" t="inlineStr">
+      <c r="M233" s="8" t="n"/>
+      <c r="N233" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13753,7 +14039,8 @@
       <c r="J234" s="8" t="n"/>
       <c r="K234" s="8" t="n"/>
       <c r="L234" s="8" t="n"/>
-      <c r="M234" s="8" t="inlineStr">
+      <c r="M234" s="8" t="n"/>
+      <c r="N234" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13808,7 +14095,8 @@
       <c r="J235" s="8" t="n"/>
       <c r="K235" s="8" t="n"/>
       <c r="L235" s="8" t="n"/>
-      <c r="M235" s="8" t="inlineStr">
+      <c r="M235" s="8" t="n"/>
+      <c r="N235" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Srixon shaft adapters' (plural) — that belongs to the Srixon adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13863,7 +14151,8 @@
       <c r="J236" s="8" t="n"/>
       <c r="K236" s="8" t="n"/>
       <c r="L236" s="8" t="n"/>
-      <c r="M236" s="8" t="inlineStr">
+      <c r="M236" s="8" t="n"/>
+      <c r="N236" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'PXG shaft adapters' (plural) — that belongs to the PXG adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13918,7 +14207,8 @@
       <c r="J237" s="8" t="n"/>
       <c r="K237" s="8" t="n"/>
       <c r="L237" s="8" t="n"/>
-      <c r="M237" s="8" t="inlineStr">
+      <c r="M237" s="8" t="n"/>
+      <c r="N237" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'PXG shaft adapters' (plural) — that belongs to the PXG adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -13973,7 +14263,8 @@
       <c r="J238" s="8" t="n"/>
       <c r="K238" s="8" t="n"/>
       <c r="L238" s="8" t="n"/>
-      <c r="M238" s="8" t="inlineStr">
+      <c r="M238" s="8" t="n"/>
+      <c r="N238" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Ping shaft adapters' (plural) — that belongs to the Ping adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14028,7 +14319,8 @@
       <c r="J239" s="8" t="n"/>
       <c r="K239" s="8" t="n"/>
       <c r="L239" s="8" t="n"/>
-      <c r="M239" s="8" t="inlineStr">
+      <c r="M239" s="8" t="n"/>
+      <c r="N239" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Ping shaft adapters' (plural) — that belongs to the Ping adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14083,7 +14375,8 @@
       <c r="J240" s="8" t="n"/>
       <c r="K240" s="8" t="n"/>
       <c r="L240" s="8" t="n"/>
-      <c r="M240" s="8" t="inlineStr">
+      <c r="M240" s="8" t="n"/>
+      <c r="N240" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'TaylorMade shaft adapters' (plural) — that belongs to the TaylorMade adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14138,7 +14431,8 @@
       <c r="J241" s="8" t="n"/>
       <c r="K241" s="8" t="n"/>
       <c r="L241" s="8" t="n"/>
-      <c r="M241" s="8" t="inlineStr">
+      <c r="M241" s="8" t="n"/>
+      <c r="N241" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Callaway shaft adapters' (plural) — that belongs to the Callaway adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14193,7 +14487,8 @@
       <c r="J242" s="8" t="n"/>
       <c r="K242" s="8" t="n"/>
       <c r="L242" s="8" t="n"/>
-      <c r="M242" s="8" t="inlineStr">
+      <c r="M242" s="8" t="n"/>
+      <c r="N242" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Callaway shaft adapters' (plural) — that belongs to the Callaway adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead. This page has an odd-looking web address — keep the URL exactly as it is (do not tidy, delete or redirect it).</t>
         </is>
@@ -14248,7 +14543,8 @@
       <c r="J243" s="8" t="n"/>
       <c r="K243" s="8" t="n"/>
       <c r="L243" s="8" t="n"/>
-      <c r="M243" s="8" t="inlineStr">
+      <c r="M243" s="8" t="n"/>
+      <c r="N243" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14303,7 +14599,8 @@
       <c r="J244" s="8" t="n"/>
       <c r="K244" s="8" t="n"/>
       <c r="L244" s="8" t="n"/>
-      <c r="M244" s="8" t="inlineStr">
+      <c r="M244" s="8" t="n"/>
+      <c r="N244" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14358,7 +14655,8 @@
       <c r="J245" s="8" t="n"/>
       <c r="K245" s="8" t="n"/>
       <c r="L245" s="8" t="n"/>
-      <c r="M245" s="8" t="inlineStr">
+      <c r="M245" s="8" t="n"/>
+      <c r="N245" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Cobra shaft adapters' (plural) — that belongs to the Cobra adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14413,7 +14711,8 @@
       <c r="J246" s="8" t="n"/>
       <c r="K246" s="8" t="n"/>
       <c r="L246" s="8" t="n"/>
-      <c r="M246" s="8" t="inlineStr">
+      <c r="M246" s="8" t="n"/>
+      <c r="N246" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Mizuno shaft adapters' (plural) — that belongs to the Mizuno adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14468,7 +14767,8 @@
       <c r="J247" s="8" t="n"/>
       <c r="K247" s="8" t="n"/>
       <c r="L247" s="8" t="n"/>
-      <c r="M247" s="8" t="inlineStr">
+      <c r="M247" s="8" t="n"/>
+      <c r="N247" s="8" t="inlineStr">
         <is>
           <t>Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14523,7 +14823,8 @@
       <c r="J248" s="8" t="n"/>
       <c r="K248" s="8" t="n"/>
       <c r="L248" s="8" t="n"/>
-      <c r="M248" s="8" t="inlineStr">
+      <c r="M248" s="8" t="n"/>
+      <c r="N248" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'PXG shaft adapters' (plural) — that belongs to the PXG adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14578,7 +14879,8 @@
       <c r="J249" s="8" t="n"/>
       <c r="K249" s="8" t="n"/>
       <c r="L249" s="8" t="n"/>
-      <c r="M249" s="8" t="inlineStr">
+      <c r="M249" s="8" t="n"/>
+      <c r="N249" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Ping shaft adapters' (plural) — that belongs to the Ping adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14633,7 +14935,8 @@
       <c r="J250" s="8" t="n"/>
       <c r="K250" s="8" t="n"/>
       <c r="L250" s="8" t="n"/>
-      <c r="M250" s="8" t="inlineStr">
+      <c r="M250" s="8" t="n"/>
+      <c r="N250" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Ping shaft adapters' (plural) — that belongs to the Ping adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14688,7 +14991,8 @@
       <c r="J251" s="8" t="n"/>
       <c r="K251" s="8" t="n"/>
       <c r="L251" s="8" t="n"/>
-      <c r="M251" s="8" t="inlineStr">
+      <c r="M251" s="8" t="n"/>
+      <c r="N251" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Ping shaft adapters' (plural) — that belongs to the Ping adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14743,7 +15047,8 @@
       <c r="J252" s="8" t="n"/>
       <c r="K252" s="8" t="n"/>
       <c r="L252" s="8" t="n"/>
-      <c r="M252" s="8" t="inlineStr">
+      <c r="M252" s="8" t="n"/>
+      <c r="N252" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Ping shaft adapters' (plural) — that belongs to the Ping adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14798,7 +15103,8 @@
       <c r="J253" s="8" t="n"/>
       <c r="K253" s="8" t="n"/>
       <c r="L253" s="8" t="n"/>
-      <c r="M253" s="8" t="inlineStr">
+      <c r="M253" s="8" t="n"/>
+      <c r="N253" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Ping shaft adapters' (plural) — that belongs to the Ping adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14853,7 +15159,8 @@
       <c r="J254" s="8" t="n"/>
       <c r="K254" s="8" t="n"/>
       <c r="L254" s="8" t="n"/>
-      <c r="M254" s="8" t="inlineStr">
+      <c r="M254" s="8" t="n"/>
+      <c r="N254" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Srixon shaft adapters' (plural) — that belongs to the Srixon adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14908,7 +15215,8 @@
       <c r="J255" s="8" t="n"/>
       <c r="K255" s="8" t="n"/>
       <c r="L255" s="8" t="n"/>
-      <c r="M255" s="8" t="inlineStr">
+      <c r="M255" s="8" t="n"/>
+      <c r="N255" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'TaylorMade shaft adapters' (plural) — that belongs to the TaylorMade adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -14963,7 +15271,8 @@
       <c r="J256" s="8" t="n"/>
       <c r="K256" s="8" t="n"/>
       <c r="L256" s="8" t="n"/>
-      <c r="M256" s="8" t="inlineStr">
+      <c r="M256" s="8" t="n"/>
+      <c r="N256" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Titleist shaft adapters' (plural) — that belongs to the Titleist adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -15018,7 +15327,8 @@
       <c r="J257" s="8" t="n"/>
       <c r="K257" s="8" t="n"/>
       <c r="L257" s="8" t="n"/>
-      <c r="M257" s="8" t="inlineStr">
+      <c r="M257" s="8" t="n"/>
+      <c r="N257" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Wilson shaft adapters' (plural) — that belongs to the Wilson adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -15073,7 +15383,8 @@
       <c r="J258" s="8" t="n"/>
       <c r="K258" s="8" t="n"/>
       <c r="L258" s="8" t="n"/>
-      <c r="M258" s="8" t="inlineStr">
+      <c r="M258" s="8" t="n"/>
+      <c r="N258" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'Wilson shaft adapters' (plural) — that belongs to the Wilson adapter collection. This page is one specific adapter. Don't add a full settings/compatibility chart here — link to the chart on the adapter collection page instead.</t>
         </is>
@@ -15097,6 +15408,7 @@
       <c r="K259" s="6" t="n"/>
       <c r="L259" s="6" t="n"/>
       <c r="M259" s="6" t="n"/>
+      <c r="N259" s="6" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="7" t="inlineStr">
@@ -15143,7 +15455,8 @@
       <c r="J260" s="8" t="n"/>
       <c r="K260" s="8" t="n"/>
       <c r="L260" s="8" t="n"/>
-      <c r="M260" s="8" t="inlineStr">
+      <c r="M260" s="8" t="n"/>
+      <c r="N260" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15194,7 +15507,8 @@
       <c r="J261" s="8" t="n"/>
       <c r="K261" s="8" t="n"/>
       <c r="L261" s="8" t="n"/>
-      <c r="M261" s="8" t="inlineStr">
+      <c r="M261" s="8" t="n"/>
+      <c r="N261" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15245,7 +15559,8 @@
       <c r="J262" s="8" t="n"/>
       <c r="K262" s="8" t="n"/>
       <c r="L262" s="8" t="n"/>
-      <c r="M262" s="8" t="inlineStr">
+      <c r="M262" s="8" t="n"/>
+      <c r="N262" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15296,7 +15611,8 @@
       <c r="J263" s="8" t="n"/>
       <c r="K263" s="8" t="n"/>
       <c r="L263" s="8" t="n"/>
-      <c r="M263" s="8" t="inlineStr">
+      <c r="M263" s="8" t="n"/>
+      <c r="N263" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15347,7 +15663,8 @@
       <c r="J264" s="8" t="n"/>
       <c r="K264" s="8" t="n"/>
       <c r="L264" s="8" t="n"/>
-      <c r="M264" s="8" t="inlineStr">
+      <c r="M264" s="8" t="n"/>
+      <c r="N264" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15398,7 +15715,8 @@
       <c r="J265" s="8" t="n"/>
       <c r="K265" s="8" t="n"/>
       <c r="L265" s="8" t="n"/>
-      <c r="M265" s="8" t="inlineStr">
+      <c r="M265" s="8" t="n"/>
+      <c r="N265" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15449,7 +15767,8 @@
       <c r="J266" s="8" t="n"/>
       <c r="K266" s="8" t="n"/>
       <c r="L266" s="8" t="n"/>
-      <c r="M266" s="8" t="inlineStr">
+      <c r="M266" s="8" t="n"/>
+      <c r="N266" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15500,7 +15819,8 @@
       <c r="J267" s="8" t="n"/>
       <c r="K267" s="8" t="n"/>
       <c r="L267" s="8" t="n"/>
-      <c r="M267" s="8" t="inlineStr">
+      <c r="M267" s="8" t="n"/>
+      <c r="N267" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15551,7 +15871,8 @@
       <c r="J268" s="8" t="n"/>
       <c r="K268" s="8" t="n"/>
       <c r="L268" s="8" t="n"/>
-      <c r="M268" s="8" t="inlineStr">
+      <c r="M268" s="8" t="n"/>
+      <c r="N268" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15602,7 +15923,8 @@
       <c r="J269" s="8" t="n"/>
       <c r="K269" s="8" t="n"/>
       <c r="L269" s="8" t="n"/>
-      <c r="M269" s="8" t="inlineStr">
+      <c r="M269" s="8" t="n"/>
+      <c r="N269" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -15653,7 +15975,8 @@
       <c r="J270" s="8" t="n"/>
       <c r="K270" s="8" t="n"/>
       <c r="L270" s="8" t="n"/>
-      <c r="M270" s="8" t="inlineStr">
+      <c r="M270" s="8" t="n"/>
+      <c r="N270" s="8" t="inlineStr">
         <is>
           <t>Don't title this page 'golf torque wrench' on its own — that phrase belongs to the Torque Wrenches collection.</t>
         </is>
@@ -17229,12 +17552,12 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>/collections/putters</t>
+          <t>/collections/drivers</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>putter head weights</t>
+          <t>driver head weights</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -17249,24 +17572,16 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>/collections/golf-club-weight-kits-1</t>
+          <t>/products/mz-aftermarket-weights-for-mizuno-st-range-drivers</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>golf club weight kits</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>/products/mz-aftermarket-weights-for-mizuno-st-range-drivers</t>
-        </is>
-      </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
           <t>Mizuno ST driver weights</t>
         </is>
       </c>
+      <c r="K21" s="8" t="n"/>
+      <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="n"/>
       <c r="N21" s="8" t="n"/>
       <c r="O21" s="8" t="n"/>
@@ -17991,7 +18306,7 @@
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>Mizuno putter weights</t>
+          <t>Mizuno golf weights</t>
         </is>
       </c>
       <c r="G34" s="8" t="n"/>

</xml_diff>